<commit_message>
Take the answers out of the practice workbook
The chronology sheet shipped with my own build notes still sitting in
its הערה column: "date as text", "same event twice", "no date in the
document". Those are exactly the four things the exercise asks the
reader to discover, and the prompt tells Claude to mark the rows
himself, so a pre-filled column both spoils the exercise and collides
with the instruction.

Column cleared. The four defects themselves are untouched and verified
still present: the two text dates, the duplicated event, the row with no
date and the missing page number.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/assets/Legal-Mind-practice-workbook.xlsx
+++ b/excel/assets/Legal-Mind-practice-workbook.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="שעות" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="שעות גרסת הצד השני" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="תעריפים" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="ציר עובדות" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="מפתח נספחים" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="תנועות בנק" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="לוח תשלומים" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="שעות" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="שעות גרסת הצד השני" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="תעריפים" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ציר עובדות" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מפתח נספחים" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="תנועות בנק" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="לוח תשלומים" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,11 +22,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
-    <numFmt numFmtId="166" formatCode="0.0"/>
-    <numFmt numFmtId="167" formatCode="#,##0&quot; ₪&quot;"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="#,##0&quot; ₪&quot;"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -91,12 +90,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -105,14 +107,21 @@
     <xf numFmtId="166" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -539,7 +548,7 @@
           <t>פלוני נ' חברת הבנייה</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n">
+      <c r="B2" s="9" t="n">
         <v>46065</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -552,13 +561,13 @@
           <t>עיון בכתב ההגנה</t>
         </is>
       </c>
-      <c r="E2" s="4" t="n">
+      <c r="E2" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="F2" s="5" t="n">
+      <c r="F2" s="11" t="n">
         <v>900</v>
       </c>
-      <c r="G2" s="5">
+      <c r="G2" s="11">
         <f>E2*F2</f>
         <v/>
       </c>
@@ -574,7 +583,7 @@
           <t>עיזבון אלמוני</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n">
+      <c r="B3" s="9" t="n">
         <v>46014</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -587,13 +596,13 @@
           <t>ישיבה עם הצד שכנגד</t>
         </is>
       </c>
-      <c r="E3" s="4" t="n">
+      <c r="E3" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="F3" s="5" t="n">
+      <c r="F3" s="11" t="n">
         <v>480</v>
       </c>
-      <c r="G3" s="5">
+      <c r="G3" s="11">
         <f>E3*F3</f>
         <v/>
       </c>
@@ -609,7 +618,7 @@
           <t>רכישת דירה ברחוב הזיתים</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="B4" s="9" t="n">
         <v>46020</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -622,13 +631,13 @@
           <t>תיאום מול השמאי</t>
         </is>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="E4" s="10" t="n">
         <v>1.5</v>
       </c>
-      <c r="F4" s="5" t="n">
+      <c r="F4" s="11" t="n">
         <v>650</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="11">
         <f>E4*F4</f>
         <v/>
       </c>
@@ -644,7 +653,7 @@
           <t>בקשה לצו מניעה</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n">
+      <c r="B5" s="9" t="n">
         <v>46081</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -657,13 +666,13 @@
           <t>מחקר פסיקה</t>
         </is>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E5" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="F5" s="5" t="n">
+      <c r="F5" s="11" t="n">
         <v>750</v>
       </c>
-      <c r="G5" s="5">
+      <c r="G5" s="11">
         <f>E5*F5</f>
         <v/>
       </c>
@@ -679,7 +688,7 @@
           <t>הסכם ממון - משפחת שרון</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B6" s="9" t="n">
         <v>46132</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -692,13 +701,13 @@
           <t>עריכת טיוטת הסכם</t>
         </is>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="E6" s="10" t="n">
         <v>2.5</v>
       </c>
-      <c r="F6" s="5" t="n">
+      <c r="F6" s="11" t="n">
         <v>900</v>
       </c>
-      <c r="G6" s="5">
+      <c r="G6" s="11">
         <f>E6*F6</f>
         <v/>
       </c>
@@ -714,7 +723,7 @@
           <t>פלוני נ' חברת הבנייה</t>
         </is>
       </c>
-      <c r="B7" s="3" t="n">
+      <c r="B7" s="9" t="n">
         <v>45981</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -727,13 +736,13 @@
           <t>שיחת ייעוץ עם הלקוח</t>
         </is>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="E7" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="F7" s="5" t="n">
+      <c r="F7" s="11" t="n">
         <v>480</v>
       </c>
-      <c r="G7" s="5">
+      <c r="G7" s="11">
         <f>E7*F7</f>
         <v/>
       </c>
@@ -749,7 +758,7 @@
           <t>עיזבון אלמוני</t>
         </is>
       </c>
-      <c r="B8" s="3" t="n">
+      <c r="B8" s="9" t="n">
         <v>46130</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -762,13 +771,13 @@
           <t>הכנה לדיון</t>
         </is>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="E8" s="10" t="n">
         <v>3.5</v>
       </c>
-      <c r="F8" s="5" t="n">
+      <c r="F8" s="11" t="n">
         <v>650</v>
       </c>
-      <c r="G8" s="5">
+      <c r="G8" s="11">
         <f>E8*F8</f>
         <v/>
       </c>
@@ -784,7 +793,7 @@
           <t>רכישת דירה ברחוב הזיתים</t>
         </is>
       </c>
-      <c r="B9" s="3" t="n">
+      <c r="B9" s="9" t="n">
         <v>46128</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -797,13 +806,13 @@
           <t>סיכום פגישה</t>
         </is>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="E9" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="F9" s="5" t="n">
+      <c r="F9" s="11" t="n">
         <v>750</v>
       </c>
-      <c r="G9" s="5">
+      <c r="G9" s="11">
         <f>E9*F9</f>
         <v/>
       </c>
@@ -819,7 +828,7 @@
           <t>בקשה לצו מניעה</t>
         </is>
       </c>
-      <c r="B10" s="3" t="n">
+      <c r="B10" s="9" t="n">
         <v>46005</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -832,13 +841,13 @@
           <t>ניסוח מכתב התראה</t>
         </is>
       </c>
-      <c r="E10" s="4" t="n">
+      <c r="E10" s="10" t="n">
         <v>4.5</v>
       </c>
-      <c r="F10" s="5" t="n">
+      <c r="F10" s="11" t="n">
         <v>900</v>
       </c>
-      <c r="G10" s="5">
+      <c r="G10" s="11">
         <f>E10*F10</f>
         <v/>
       </c>
@@ -854,7 +863,7 @@
           <t>הסכם ממון - משפחת שרון</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n">
+      <c r="B11" s="9" t="n">
         <v>46020</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -867,13 +876,13 @@
           <t>בדיקת נסח טאבו</t>
         </is>
       </c>
-      <c r="E11" s="4" t="n">
+      <c r="E11" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="F11" s="5" t="n">
+      <c r="F11" s="11" t="n">
         <v>480</v>
       </c>
-      <c r="G11" s="5">
+      <c r="G11" s="11">
         <f>E11*F11</f>
         <v/>
       </c>
@@ -889,7 +898,7 @@
           <t>פלוני נ' חברת הבנייה</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n">
+      <c r="B12" s="9" t="n">
         <v>46022</v>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -902,13 +911,13 @@
           <t>הכנת תצהיר</t>
         </is>
       </c>
-      <c r="E12" s="4" t="n">
+      <c r="E12" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="F12" s="5" t="n">
+      <c r="F12" s="11" t="n">
         <v>650</v>
       </c>
-      <c r="G12" s="5">
+      <c r="G12" s="11">
         <f>E12*F12</f>
         <v/>
       </c>
@@ -924,7 +933,7 @@
           <t>עיזבון אלמוני</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>3.12.2025</t>
         </is>
@@ -939,13 +948,13 @@
           <t>דיון בבית המשפט</t>
         </is>
       </c>
-      <c r="E13" s="4" t="n">
+      <c r="E13" s="10" t="n">
         <v>1.5</v>
       </c>
-      <c r="F13" s="5" t="n">
+      <c r="F13" s="11" t="n">
         <v>750</v>
       </c>
-      <c r="G13" s="5">
+      <c r="G13" s="11">
         <f>E13*F13</f>
         <v/>
       </c>
@@ -961,7 +970,7 @@
           <t>רכישת דירה ברחוב הזיתים</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n">
+      <c r="B14" s="9" t="n">
         <v>46117</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -974,13 +983,13 @@
           <t>עיון בכתב ההגנה</t>
         </is>
       </c>
-      <c r="E14" s="4" t="n">
+      <c r="E14" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="F14" s="5" t="n">
+      <c r="F14" s="11" t="n">
         <v>900</v>
       </c>
-      <c r="G14" s="5">
+      <c r="G14" s="11">
         <f>E14*F14</f>
         <v/>
       </c>
@@ -996,7 +1005,7 @@
           <t>בקשה לצו מניעה</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n">
+      <c r="B15" s="9" t="n">
         <v>46098</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1009,13 +1018,13 @@
           <t>ישיבה עם הצד שכנגד</t>
         </is>
       </c>
-      <c r="E15" s="4" t="n">
+      <c r="E15" s="10" t="n">
         <v>2.5</v>
       </c>
-      <c r="F15" s="5" t="n">
+      <c r="F15" s="11" t="n">
         <v>480</v>
       </c>
-      <c r="G15" s="5">
+      <c r="G15" s="11">
         <f>E15*F15</f>
         <v/>
       </c>
@@ -1031,7 +1040,7 @@
           <t>הסכם ממון - משפחת שרון</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n">
+      <c r="B16" s="9" t="n">
         <v>45967</v>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1044,13 +1053,13 @@
           <t>תיאום מול השמאי</t>
         </is>
       </c>
-      <c r="E16" s="4" t="n">
+      <c r="E16" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="F16" s="5" t="n">
+      <c r="F16" s="11" t="n">
         <v>650</v>
       </c>
-      <c r="G16" s="5">
+      <c r="G16" s="11">
         <f>E16*F16</f>
         <v/>
       </c>
@@ -1066,7 +1075,7 @@
           <t>פלוני נ' חברת הבנייה</t>
         </is>
       </c>
-      <c r="B17" s="3" t="n">
+      <c r="B17" s="9" t="n">
         <v>45965</v>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1079,13 +1088,13 @@
           <t>מחקר פסיקה</t>
         </is>
       </c>
-      <c r="E17" s="4" t="n">
+      <c r="E17" s="10" t="n">
         <v>3.5</v>
       </c>
-      <c r="F17" s="5" t="n">
+      <c r="F17" s="11" t="n">
         <v>750</v>
       </c>
-      <c r="G17" s="5">
+      <c r="G17" s="11">
         <f>E17*F17</f>
         <v/>
       </c>
@@ -1101,7 +1110,7 @@
           <t>עיזבון אלמוני</t>
         </is>
       </c>
-      <c r="B18" s="3" t="n">
+      <c r="B18" s="9" t="n">
         <v>46037</v>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1114,13 +1123,13 @@
           <t>עריכת טיוטת הסכם</t>
         </is>
       </c>
-      <c r="E18" s="4" t="n">
+      <c r="E18" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="F18" s="5" t="n">
+      <c r="F18" s="11" t="n">
         <v>900</v>
       </c>
-      <c r="G18" s="5">
+      <c r="G18" s="11">
         <f>E18*F18</f>
         <v/>
       </c>
@@ -1136,7 +1145,7 @@
           <t>רכישת דירה ברחוב הזיתים</t>
         </is>
       </c>
-      <c r="B19" s="3" t="n">
+      <c r="B19" s="9" t="n">
         <v>46086</v>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -1149,13 +1158,13 @@
           <t>שיחת ייעוץ עם הלקוח</t>
         </is>
       </c>
-      <c r="E19" s="4" t="n">
+      <c r="E19" s="10" t="n">
         <v>4.5</v>
       </c>
-      <c r="F19" s="5" t="n">
+      <c r="F19" s="11" t="n">
         <v>480</v>
       </c>
-      <c r="G19" s="5">
+      <c r="G19" s="11">
         <f>E19*F19</f>
         <v/>
       </c>
@@ -1171,7 +1180,7 @@
           <t>בקשה לצו מניעה</t>
         </is>
       </c>
-      <c r="B20" s="3" t="n">
+      <c r="B20" s="9" t="n">
         <v>46063</v>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1184,13 +1193,13 @@
           <t>הכנה לדיון</t>
         </is>
       </c>
-      <c r="E20" s="4" t="n">
+      <c r="E20" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="F20" s="5" t="n">
+      <c r="F20" s="11" t="n">
         <v>650</v>
       </c>
-      <c r="G20" s="5">
+      <c r="G20" s="11">
         <f>E20*F20</f>
         <v/>
       </c>
@@ -1206,7 +1215,7 @@
           <t>הסכם ממון - משפחת שרון</t>
         </is>
       </c>
-      <c r="B21" s="3" t="n">
+      <c r="B21" s="9" t="n">
         <v>46002</v>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -1219,13 +1228,13 @@
           <t>סיכום פגישה</t>
         </is>
       </c>
-      <c r="E21" s="4" t="n">
+      <c r="E21" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="F21" s="5" t="n">
+      <c r="F21" s="11" t="n">
         <v>750</v>
       </c>
-      <c r="G21" s="5">
+      <c r="G21" s="11">
         <f>E21*F21</f>
         <v/>
       </c>
@@ -1241,7 +1250,7 @@
           <t>פלוני נ' חברת הבנייה</t>
         </is>
       </c>
-      <c r="B22" s="3" t="n">
+      <c r="B22" s="9" t="n">
         <v>45965</v>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1254,13 +1263,13 @@
           <t>ניסוח מכתב התראה</t>
         </is>
       </c>
-      <c r="E22" s="4" t="n">
+      <c r="E22" s="10" t="n">
         <v>1.5</v>
       </c>
-      <c r="F22" s="5" t="n">
+      <c r="F22" s="11" t="n">
         <v>900</v>
       </c>
-      <c r="G22" s="5">
+      <c r="G22" s="11">
         <f>E22*F22</f>
         <v/>
       </c>
@@ -1276,7 +1285,7 @@
           <t>עיזבון אלמוני</t>
         </is>
       </c>
-      <c r="B23" s="3" t="n">
+      <c r="B23" s="9" t="n">
         <v>46059</v>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -1289,13 +1298,13 @@
           <t>בדיקת נסח טאבו</t>
         </is>
       </c>
-      <c r="E23" s="4" t="n">
+      <c r="E23" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="F23" s="5" t="n">
+      <c r="F23" s="11" t="n">
         <v>480</v>
       </c>
-      <c r="G23" s="5">
+      <c r="G23" s="11">
         <f>E23*F23</f>
         <v/>
       </c>
@@ -1311,7 +1320,7 @@
           <t>רכישת דירה ברחוב הזיתים</t>
         </is>
       </c>
-      <c r="B24" s="3" t="n">
+      <c r="B24" s="9" t="n">
         <v>45990</v>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -1324,13 +1333,13 @@
           <t>הכנת תצהיר</t>
         </is>
       </c>
-      <c r="E24" s="4" t="n">
+      <c r="E24" s="10" t="n">
         <v>2.5</v>
       </c>
-      <c r="F24" s="5" t="n">
+      <c r="F24" s="11" t="n">
         <v>650</v>
       </c>
-      <c r="G24" s="5">
+      <c r="G24" s="11">
         <f>E24*F24</f>
         <v/>
       </c>
@@ -1346,7 +1355,7 @@
           <t>בקשה לצו מניעה</t>
         </is>
       </c>
-      <c r="B25" s="3" t="n">
+      <c r="B25" s="9" t="n">
         <v>46117</v>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -1359,13 +1368,13 @@
           <t>דיון בבית המשפט</t>
         </is>
       </c>
-      <c r="E25" s="4" t="n">
+      <c r="E25" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="F25" s="5" t="n">
+      <c r="F25" s="11" t="n">
         <v>750</v>
       </c>
-      <c r="G25" s="5">
+      <c r="G25" s="11">
         <f>E25*F25</f>
         <v/>
       </c>
@@ -1381,7 +1390,7 @@
           <t>הסכם ממון - משפחת שרון</t>
         </is>
       </c>
-      <c r="B26" s="3" t="n">
+      <c r="B26" s="9" t="n">
         <v>46057</v>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1394,13 +1403,13 @@
           <t>עיון בכתב ההגנה</t>
         </is>
       </c>
-      <c r="E26" s="4" t="n">
+      <c r="E26" s="10" t="n">
         <v>3.5</v>
       </c>
-      <c r="F26" s="5" t="n">
+      <c r="F26" s="11" t="n">
         <v>900</v>
       </c>
-      <c r="G26" s="5">
+      <c r="G26" s="11">
         <f>E26*F26</f>
         <v/>
       </c>
@@ -1416,7 +1425,7 @@
           <t>פלוני נ' חברת הבנייה</t>
         </is>
       </c>
-      <c r="B27" s="3" t="n">
+      <c r="B27" s="9" t="n">
         <v>46039</v>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -1429,13 +1438,13 @@
           <t>ישיבה עם הצד שכנגד</t>
         </is>
       </c>
-      <c r="E27" s="4" t="n">
+      <c r="E27" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="F27" s="5" t="n">
+      <c r="F27" s="11" t="n">
         <v>480</v>
       </c>
-      <c r="G27" s="5">
+      <c r="G27" s="11">
         <f>E27*F27</f>
         <v/>
       </c>
@@ -1451,7 +1460,7 @@
           <t>עיזבון אלמוני</t>
         </is>
       </c>
-      <c r="B28" s="3" t="n">
+      <c r="B28" s="9" t="n">
         <v>46128</v>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -1464,13 +1473,13 @@
           <t>תיאום מול השמאי</t>
         </is>
       </c>
-      <c r="E28" s="4" t="n">
+      <c r="E28" s="10" t="n">
         <v>4.5</v>
       </c>
-      <c r="F28" s="5" t="n">
+      <c r="F28" s="11" t="n">
         <v>650</v>
       </c>
-      <c r="G28" s="5">
+      <c r="G28" s="11">
         <f>E28*F28</f>
         <v/>
       </c>
@@ -1486,7 +1495,7 @@
           <t>רכישת דירה ברחוב הזיתים</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B29" s="9" t="inlineStr">
         <is>
           <t>2026-01-14</t>
         </is>
@@ -1501,13 +1510,13 @@
           <t>מחקר פסיקה</t>
         </is>
       </c>
-      <c r="E29" s="4" t="n">
+      <c r="E29" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="F29" s="5" t="n">
+      <c r="F29" s="11" t="n">
         <v>750</v>
       </c>
-      <c r="G29" s="5">
+      <c r="G29" s="11">
         <f>E29*F29</f>
         <v/>
       </c>
@@ -1523,7 +1532,7 @@
           <t>בקשה לצו מניעה</t>
         </is>
       </c>
-      <c r="B30" s="3" t="n">
+      <c r="B30" s="9" t="n">
         <v>46101</v>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -1536,13 +1545,13 @@
           <t>עריכת טיוטת הסכם</t>
         </is>
       </c>
-      <c r="E30" s="4" t="n">
+      <c r="E30" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="F30" s="5" t="n">
+      <c r="F30" s="11" t="n">
         <v>900</v>
       </c>
-      <c r="G30" s="5">
+      <c r="G30" s="11">
         <f>E30*F30</f>
         <v/>
       </c>
@@ -1558,7 +1567,7 @@
           <t>הסכם ממון - משפחת שרון</t>
         </is>
       </c>
-      <c r="B31" s="3" t="n">
+      <c r="B31" s="9" t="n">
         <v>46042</v>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -1571,13 +1580,13 @@
           <t>שיחת ייעוץ עם הלקוח</t>
         </is>
       </c>
-      <c r="E31" s="4" t="n">
+      <c r="E31" s="10" t="n">
         <v>1.5</v>
       </c>
-      <c r="F31" s="5" t="n">
+      <c r="F31" s="11" t="n">
         <v>480</v>
       </c>
-      <c r="G31" s="5">
+      <c r="G31" s="11">
         <f>E31*F31</f>
         <v/>
       </c>
@@ -1593,7 +1602,7 @@
           <t>פלוני נ' חברת הבנייה</t>
         </is>
       </c>
-      <c r="B32" s="3" t="n">
+      <c r="B32" s="9" t="n">
         <v>46036</v>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -1606,13 +1615,13 @@
           <t>הכנה לדיון</t>
         </is>
       </c>
-      <c r="E32" s="4" t="n">
+      <c r="E32" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="F32" s="5" t="n">
+      <c r="F32" s="11" t="n">
         <v>650</v>
       </c>
-      <c r="G32" s="5">
+      <c r="G32" s="11">
         <f>E32*F32</f>
         <v/>
       </c>
@@ -1628,7 +1637,7 @@
           <t>עיזבון אלמוני</t>
         </is>
       </c>
-      <c r="B33" s="3" t="n">
+      <c r="B33" s="9" t="n">
         <v>46030</v>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -1641,13 +1650,13 @@
           <t>סיכום פגישה</t>
         </is>
       </c>
-      <c r="E33" s="4" t="n">
+      <c r="E33" s="10" t="n">
         <v>2.5</v>
       </c>
-      <c r="F33" s="5" t="n">
+      <c r="F33" s="11" t="n">
         <v>750</v>
       </c>
-      <c r="G33" s="5">
+      <c r="G33" s="11">
         <f>E33*F33</f>
         <v/>
       </c>
@@ -1663,7 +1672,7 @@
           <t>רכישת דירה ברחוב הזיתים</t>
         </is>
       </c>
-      <c r="B34" s="3" t="n">
+      <c r="B34" s="9" t="n">
         <v>46103</v>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -1676,13 +1685,13 @@
           <t>ניסוח מכתב התראה</t>
         </is>
       </c>
-      <c r="E34" s="4" t="n">
+      <c r="E34" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="F34" s="5" t="n">
+      <c r="F34" s="11" t="n">
         <v>900</v>
       </c>
-      <c r="G34" s="5">
+      <c r="G34" s="11">
         <f>E34*F34</f>
         <v/>
       </c>
@@ -1698,7 +1707,7 @@
           <t>בקשה לצו מניעה</t>
         </is>
       </c>
-      <c r="B35" s="3" t="n">
+      <c r="B35" s="9" t="n">
         <v>45987</v>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -1711,15 +1720,15 @@
           <t>בדיקת נסח טאבו</t>
         </is>
       </c>
-      <c r="E35" s="4" t="inlineStr">
+      <c r="E35" s="10" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F35" s="5" t="n">
+      <c r="F35" s="11" t="n">
         <v>480</v>
       </c>
-      <c r="G35" s="5">
+      <c r="G35" s="11">
         <f>E35*F35</f>
         <v/>
       </c>
@@ -1735,7 +1744,7 @@
           <t>הסכם ממון - משפחת שרון</t>
         </is>
       </c>
-      <c r="B36" s="3" t="n">
+      <c r="B36" s="9" t="n">
         <v>46105</v>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -1748,13 +1757,13 @@
           <t>הכנת תצהיר</t>
         </is>
       </c>
-      <c r="E36" s="4" t="n">
+      <c r="E36" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="F36" s="5" t="n">
+      <c r="F36" s="11" t="n">
         <v>650</v>
       </c>
-      <c r="G36" s="5">
+      <c r="G36" s="11">
         <f>E36*F36</f>
         <v/>
       </c>
@@ -1770,7 +1779,7 @@
           <t>פלוני נ' חברת הבנייה</t>
         </is>
       </c>
-      <c r="B37" s="3" t="n">
+      <c r="B37" s="9" t="n">
         <v>46088</v>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -1783,13 +1792,13 @@
           <t>דיון בבית המשפט</t>
         </is>
       </c>
-      <c r="E37" s="4" t="n">
+      <c r="E37" s="10" t="n">
         <v>4.5</v>
       </c>
-      <c r="F37" s="5" t="n">
+      <c r="F37" s="11" t="n">
         <v>750</v>
       </c>
-      <c r="G37" s="5">
+      <c r="G37" s="11">
         <f>E37*F37</f>
         <v/>
       </c>
@@ -1805,7 +1814,7 @@
           <t>עיזבון אלמוני</t>
         </is>
       </c>
-      <c r="B38" s="3" t="n">
+      <c r="B38" s="9" t="n">
         <v>46071</v>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -1818,13 +1827,13 @@
           <t>עיון בכתב ההגנה</t>
         </is>
       </c>
-      <c r="E38" s="4" t="n">
+      <c r="E38" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="F38" s="5" t="n">
+      <c r="F38" s="11" t="n">
         <v>900</v>
       </c>
-      <c r="G38" s="5">
+      <c r="G38" s="11">
         <f>E38*F38</f>
         <v/>
       </c>
@@ -1840,7 +1849,7 @@
           <t>רכישת דירה ברחוב הזיתים</t>
         </is>
       </c>
-      <c r="B39" s="3" t="n">
+      <c r="B39" s="9" t="n">
         <v>45981</v>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -1853,13 +1862,13 @@
           <t>ישיבה עם הצד שכנגד</t>
         </is>
       </c>
-      <c r="E39" s="4" t="n">
+      <c r="E39" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="F39" s="5" t="n">
+      <c r="F39" s="11" t="n">
         <v>480</v>
       </c>
-      <c r="G39" s="5">
+      <c r="G39" s="11">
         <f>E39*F39</f>
         <v/>
       </c>
@@ -1875,7 +1884,7 @@
           <t>בקשה לצו מניעה</t>
         </is>
       </c>
-      <c r="B40" s="3" t="n">
+      <c r="B40" s="9" t="n">
         <v>46016</v>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -1888,13 +1897,13 @@
           <t>תיאום מול השמאי</t>
         </is>
       </c>
-      <c r="E40" s="4" t="n">
+      <c r="E40" s="10" t="n">
         <v>1.5</v>
       </c>
-      <c r="F40" s="5" t="n">
+      <c r="F40" s="11" t="n">
         <v>650</v>
       </c>
-      <c r="G40" s="5">
+      <c r="G40" s="11">
         <f>E40*F40</f>
         <v/>
       </c>
@@ -1910,7 +1919,7 @@
           <t>הסכם ממון - משפחת שרון</t>
         </is>
       </c>
-      <c r="B41" s="3" t="n">
+      <c r="B41" s="9" t="n">
         <v>46119</v>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -1923,13 +1932,13 @@
           <t>מחקר פסיקה</t>
         </is>
       </c>
-      <c r="E41" s="4" t="n">
+      <c r="E41" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="F41" s="5" t="n">
+      <c r="F41" s="11" t="n">
         <v>750</v>
       </c>
-      <c r="G41" s="5">
+      <c r="G41" s="11">
         <f>E41*F41</f>
         <v/>
       </c>
@@ -1945,7 +1954,7 @@
           <t>פלוני נ' חברת הבנייה</t>
         </is>
       </c>
-      <c r="B42" s="3" t="n">
+      <c r="B42" s="9" t="n">
         <v>46068</v>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -1958,13 +1967,13 @@
           <t>עריכת טיוטת הסכם</t>
         </is>
       </c>
-      <c r="E42" s="4" t="n">
+      <c r="E42" s="10" t="n">
         <v>2.5</v>
       </c>
-      <c r="F42" s="5" t="n">
+      <c r="F42" s="11" t="n">
         <v>900</v>
       </c>
-      <c r="G42" s="5">
+      <c r="G42" s="11">
         <f>E42*F42</f>
         <v/>
       </c>
@@ -1980,7 +1989,7 @@
           <t>עיזבון אלמוני</t>
         </is>
       </c>
-      <c r="B43" s="3" t="n">
+      <c r="B43" s="9" t="n">
         <v>46034</v>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -1993,11 +2002,11 @@
           <t>שיחת ייעוץ עם הלקוח</t>
         </is>
       </c>
-      <c r="E43" s="4" t="n">
+      <c r="E43" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="F43" s="5" t="n"/>
-      <c r="G43" s="5">
+      <c r="F43" s="11" t="n"/>
+      <c r="G43" s="11">
         <f>E43*F43</f>
         <v/>
       </c>
@@ -2013,7 +2022,7 @@
           <t>רכישת דירה ברחוב הזיתים</t>
         </is>
       </c>
-      <c r="B44" s="3" t="n">
+      <c r="B44" s="9" t="n">
         <v>45968</v>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2026,13 +2035,13 @@
           <t>הכנה לדיון</t>
         </is>
       </c>
-      <c r="E44" s="4" t="n">
+      <c r="E44" s="10" t="n">
         <v>3.5</v>
       </c>
-      <c r="F44" s="5" t="n">
+      <c r="F44" s="11" t="n">
         <v>650</v>
       </c>
-      <c r="G44" s="5">
+      <c r="G44" s="11">
         <f>E44*F44</f>
         <v/>
       </c>
@@ -2048,7 +2057,7 @@
           <t>בקשה לצו מניעה</t>
         </is>
       </c>
-      <c r="B45" s="3" t="n">
+      <c r="B45" s="9" t="n">
         <v>46113</v>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -2061,13 +2070,13 @@
           <t>סיכום פגישה</t>
         </is>
       </c>
-      <c r="E45" s="4" t="n">
+      <c r="E45" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="F45" s="5" t="n">
+      <c r="F45" s="11" t="n">
         <v>750</v>
       </c>
-      <c r="G45" s="5">
+      <c r="G45" s="11">
         <f>E45*F45</f>
         <v/>
       </c>
@@ -2083,7 +2092,7 @@
           <t>הסכם ממון - משפחת שרון</t>
         </is>
       </c>
-      <c r="B46" s="3" t="n">
+      <c r="B46" s="9" t="n">
         <v>45989</v>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -2096,13 +2105,13 @@
           <t>ניסוח מכתב התראה</t>
         </is>
       </c>
-      <c r="E46" s="4" t="n">
+      <c r="E46" s="10" t="n">
         <v>4.5</v>
       </c>
-      <c r="F46" s="5" t="n">
+      <c r="F46" s="11" t="n">
         <v>900</v>
       </c>
-      <c r="G46" s="5">
+      <c r="G46" s="11">
         <f>E46*F46</f>
         <v/>
       </c>
@@ -2118,7 +2127,7 @@
           <t>הסכם ממון - משפחת שרון</t>
         </is>
       </c>
-      <c r="B47" s="3" t="n">
+      <c r="B47" s="9" t="n">
         <v>45989</v>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -2131,13 +2140,13 @@
           <t>ניסוח מכתב התראה</t>
         </is>
       </c>
-      <c r="E47" s="4" t="n">
+      <c r="E47" s="10" t="n">
         <v>4.5</v>
       </c>
-      <c r="F47" s="5" t="n">
+      <c r="F47" s="11" t="n">
         <v>900</v>
       </c>
-      <c r="G47" s="5">
+      <c r="G47" s="11">
         <f>E47*F47</f>
         <v/>
       </c>
@@ -2153,7 +2162,7 @@
           <t>פלוני נ' חברת הבנייה</t>
         </is>
       </c>
-      <c r="B48" s="3" t="n">
+      <c r="B48" s="9" t="n">
         <v>46045</v>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -2166,13 +2175,13 @@
           <t>בדיקת נסח טאבו</t>
         </is>
       </c>
-      <c r="E48" s="4" t="n">
+      <c r="E48" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="F48" s="5" t="n">
+      <c r="F48" s="11" t="n">
         <v>480</v>
       </c>
-      <c r="G48" s="5">
+      <c r="G48" s="11">
         <f>E48*F48</f>
         <v/>
       </c>
@@ -2188,7 +2197,7 @@
           <t>עיזבון אלמוני</t>
         </is>
       </c>
-      <c r="B49" s="3" t="n">
+      <c r="B49" s="9" t="n">
         <v>46033</v>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -2201,13 +2210,13 @@
           <t>הכנת תצהיר</t>
         </is>
       </c>
-      <c r="E49" s="4" t="n">
+      <c r="E49" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="F49" s="5" t="n">
+      <c r="F49" s="11" t="n">
         <v>650</v>
       </c>
-      <c r="G49" s="5">
+      <c r="G49" s="11">
         <f>E49*F49</f>
         <v/>
       </c>
@@ -2223,7 +2232,7 @@
           <t>רכישת דירה ברחוב הזיתים</t>
         </is>
       </c>
-      <c r="B50" s="3" t="n">
+      <c r="B50" s="9" t="n">
         <v>46000</v>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -2236,13 +2245,13 @@
           <t>דיון בבית המשפט</t>
         </is>
       </c>
-      <c r="E50" s="4" t="n">
+      <c r="E50" s="10" t="n">
         <v>1.5</v>
       </c>
-      <c r="F50" s="5" t="n">
+      <c r="F50" s="11" t="n">
         <v>750</v>
       </c>
-      <c r="G50" s="5">
+      <c r="G50" s="11">
         <f>E50*F50</f>
         <v/>
       </c>
@@ -2258,7 +2267,7 @@
           <t>בקשה לצו מניעה</t>
         </is>
       </c>
-      <c r="B51" s="3" t="n">
+      <c r="B51" s="9" t="n">
         <v>45992</v>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -2271,13 +2280,13 @@
           <t>עיון בכתב ההגנה</t>
         </is>
       </c>
-      <c r="E51" s="4" t="n">
+      <c r="E51" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="F51" s="5" t="n">
+      <c r="F51" s="11" t="n">
         <v>900</v>
       </c>
-      <c r="G51" s="5">
+      <c r="G51" s="11">
         <f>E51*F51</f>
         <v/>
       </c>
@@ -2293,7 +2302,7 @@
           <t>הסכם ממון - משפחת שרון</t>
         </is>
       </c>
-      <c r="B52" s="3" t="n">
+      <c r="B52" s="9" t="n">
         <v>45982</v>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -2306,13 +2315,13 @@
           <t>ישיבה עם הצד שכנגד</t>
         </is>
       </c>
-      <c r="E52" s="4" t="n">
+      <c r="E52" s="10" t="n">
         <v>2.5</v>
       </c>
-      <c r="F52" s="5" t="n">
+      <c r="F52" s="11" t="n">
         <v>480</v>
       </c>
-      <c r="G52" s="5">
+      <c r="G52" s="11">
         <f>E52*F52</f>
         <v/>
       </c>
@@ -2328,7 +2337,7 @@
           <t>פלוני נ' חברת הבנייה</t>
         </is>
       </c>
-      <c r="B53" s="3" t="n">
+      <c r="B53" s="9" t="n">
         <v>46010</v>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -2341,13 +2350,13 @@
           <t>תיאום מול השמאי</t>
         </is>
       </c>
-      <c r="E53" s="4" t="n">
+      <c r="E53" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="F53" s="5" t="n">
+      <c r="F53" s="11" t="n">
         <v>650</v>
       </c>
-      <c r="G53" s="5">
+      <c r="G53" s="11">
         <f>E53*F53</f>
         <v/>
       </c>
@@ -2363,7 +2372,7 @@
           <t>עיזבון אלמוני</t>
         </is>
       </c>
-      <c r="B54" s="3" t="n">
+      <c r="B54" s="9" t="n">
         <v>46102</v>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -2376,13 +2385,13 @@
           <t>מחקר פסיקה</t>
         </is>
       </c>
-      <c r="E54" s="4" t="n">
+      <c r="E54" s="10" t="n">
         <v>3.5</v>
       </c>
-      <c r="F54" s="5" t="n">
+      <c r="F54" s="11" t="n">
         <v>750</v>
       </c>
-      <c r="G54" s="5">
+      <c r="G54" s="11">
         <f>E54*F54</f>
         <v/>
       </c>
@@ -2398,7 +2407,7 @@
           <t>רכישת דירה ברחוב הזיתים</t>
         </is>
       </c>
-      <c r="B55" s="3" t="n">
+      <c r="B55" s="9" t="n">
         <v>46004</v>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -2411,13 +2420,13 @@
           <t>עריכת טיוטת הסכם</t>
         </is>
       </c>
-      <c r="E55" s="4" t="n">
+      <c r="E55" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="F55" s="5" t="n">
+      <c r="F55" s="11" t="n">
         <v>900</v>
       </c>
-      <c r="G55" s="5">
+      <c r="G55" s="11">
         <f>E55*F55</f>
         <v/>
       </c>
@@ -2433,7 +2442,7 @@
           <t>בקשה לצו מניעה</t>
         </is>
       </c>
-      <c r="B56" s="3" t="n">
+      <c r="B56" s="9" t="n">
         <v>46063</v>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -2446,13 +2455,13 @@
           <t>שיחת ייעוץ עם הלקוח</t>
         </is>
       </c>
-      <c r="E56" s="4" t="n">
+      <c r="E56" s="10" t="n">
         <v>4.5</v>
       </c>
-      <c r="F56" s="5" t="n">
+      <c r="F56" s="11" t="n">
         <v>480</v>
       </c>
-      <c r="G56" s="5">
+      <c r="G56" s="11">
         <f>E56*F56</f>
         <v/>
       </c>
@@ -2468,7 +2477,7 @@
           <t>הסכם ממון - משפחת שרון</t>
         </is>
       </c>
-      <c r="B57" s="3" t="n">
+      <c r="B57" s="9" t="n">
         <v>46066</v>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -2481,13 +2490,13 @@
           <t>הכנה לדיון</t>
         </is>
       </c>
-      <c r="E57" s="4" t="n">
+      <c r="E57" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="F57" s="5" t="n">
+      <c r="F57" s="11" t="n">
         <v>650</v>
       </c>
-      <c r="G57" s="5">
+      <c r="G57" s="11">
         <f>E57*F57</f>
         <v/>
       </c>
@@ -2503,7 +2512,7 @@
           <t>פלוני נ' חברת הבנייה</t>
         </is>
       </c>
-      <c r="B58" s="3" t="n">
+      <c r="B58" s="9" t="n">
         <v>46113</v>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -2516,13 +2525,13 @@
           <t>סיכום פגישה</t>
         </is>
       </c>
-      <c r="E58" s="4" t="n">
+      <c r="E58" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="F58" s="5" t="n">
+      <c r="F58" s="11" t="n">
         <v>750</v>
       </c>
-      <c r="G58" s="5">
+      <c r="G58" s="11">
         <f>E58*F58</f>
         <v/>
       </c>
@@ -2538,7 +2547,7 @@
           <t>עיזבון אלמוני</t>
         </is>
       </c>
-      <c r="B59" s="3" t="n">
+      <c r="B59" s="9" t="n">
         <v>46073</v>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -2551,13 +2560,13 @@
           <t>ניסוח מכתב התראה</t>
         </is>
       </c>
-      <c r="E59" s="4" t="n">
+      <c r="E59" s="10" t="n">
         <v>1.5</v>
       </c>
-      <c r="F59" s="5" t="n">
+      <c r="F59" s="11" t="n">
         <v>900</v>
       </c>
-      <c r="G59" s="5">
+      <c r="G59" s="11">
         <f>E59*F59</f>
         <v/>
       </c>
@@ -2573,7 +2582,7 @@
           <t>רכישת דירה ברחוב הזיתים</t>
         </is>
       </c>
-      <c r="B60" s="3" t="n">
+      <c r="B60" s="9" t="n">
         <v>46020</v>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -2586,13 +2595,13 @@
           <t>בדיקת נסח טאבו</t>
         </is>
       </c>
-      <c r="E60" s="4" t="n">
+      <c r="E60" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="F60" s="5" t="n">
+      <c r="F60" s="11" t="n">
         <v>480</v>
       </c>
-      <c r="G60" s="5">
+      <c r="G60" s="11">
         <f>E60*F60</f>
         <v/>
       </c>
@@ -2608,7 +2617,7 @@
           <t>סך הכל</t>
         </is>
       </c>
-      <c r="G62" s="7">
+      <c r="G62" s="12">
         <f>SUM(G2:G60)</f>
         <v/>
       </c>
@@ -2679,7 +2688,7 @@
           <t>פלוני נ' חברת הבנייה</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n">
+      <c r="B2" s="9" t="n">
         <v>46065</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -2692,13 +2701,13 @@
           <t>עיון בכתב ההגנה</t>
         </is>
       </c>
-      <c r="E2" s="4" t="n">
+      <c r="E2" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="F2" s="5" t="n">
+      <c r="F2" s="11" t="n">
         <v>900</v>
       </c>
-      <c r="G2" s="5">
+      <c r="G2" s="11">
         <f>E2*F2</f>
         <v/>
       </c>
@@ -2709,7 +2718,7 @@
           <t>עיזבון אלמוני</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n">
+      <c r="B3" s="9" t="n">
         <v>46014</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -2722,13 +2731,13 @@
           <t>ישיבה עם הצד שכנגד</t>
         </is>
       </c>
-      <c r="E3" s="4" t="n">
+      <c r="E3" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="F3" s="5" t="n">
+      <c r="F3" s="11" t="n">
         <v>480</v>
       </c>
-      <c r="G3" s="5">
+      <c r="G3" s="11">
         <f>E3*F3</f>
         <v/>
       </c>
@@ -2739,7 +2748,7 @@
           <t>רכישת דירה ברחוב הזיתים</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="B4" s="9" t="n">
         <v>46020</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -2752,13 +2761,13 @@
           <t>תיאום מול השמאי</t>
         </is>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="E4" s="10" t="n">
         <v>1.5</v>
       </c>
-      <c r="F4" s="5" t="n">
+      <c r="F4" s="11" t="n">
         <v>650</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="11">
         <f>E4*F4</f>
         <v/>
       </c>
@@ -2769,7 +2778,7 @@
           <t>בקשה לצו מניעה</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n">
+      <c r="B5" s="9" t="n">
         <v>46081</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -2782,13 +2791,13 @@
           <t>מחקר פסיקה</t>
         </is>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E5" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="F5" s="5" t="n">
+      <c r="F5" s="11" t="n">
         <v>750</v>
       </c>
-      <c r="G5" s="5">
+      <c r="G5" s="11">
         <f>E5*F5</f>
         <v/>
       </c>
@@ -2799,7 +2808,7 @@
           <t>הסכם ממון - משפחת שרון</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B6" s="9" t="n">
         <v>46132</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -2812,13 +2821,13 @@
           <t>עריכת טיוטת הסכם</t>
         </is>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="E6" s="10" t="n">
         <v>2.5</v>
       </c>
-      <c r="F6" s="5" t="n">
+      <c r="F6" s="11" t="n">
         <v>900</v>
       </c>
-      <c r="G6" s="5">
+      <c r="G6" s="11">
         <f>E6*F6</f>
         <v/>
       </c>
@@ -2829,7 +2838,7 @@
           <t>פלוני נ' חברת הבנייה</t>
         </is>
       </c>
-      <c r="B7" s="3" t="n">
+      <c r="B7" s="9" t="n">
         <v>45981</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -2842,13 +2851,13 @@
           <t>שיחת ייעוץ עם הלקוח</t>
         </is>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="E7" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="F7" s="5" t="n">
+      <c r="F7" s="11" t="n">
         <v>480</v>
       </c>
-      <c r="G7" s="5">
+      <c r="G7" s="11">
         <f>E7*F7</f>
         <v/>
       </c>
@@ -2859,7 +2868,7 @@
           <t>עיזבון אלמוני</t>
         </is>
       </c>
-      <c r="B8" s="3" t="n">
+      <c r="B8" s="9" t="n">
         <v>46130</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -2872,13 +2881,13 @@
           <t>הכנה לדיון</t>
         </is>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="E8" s="10" t="n">
         <v>3.5</v>
       </c>
-      <c r="F8" s="5" t="n">
+      <c r="F8" s="11" t="n">
         <v>650</v>
       </c>
-      <c r="G8" s="5">
+      <c r="G8" s="11">
         <f>E8*F8</f>
         <v/>
       </c>
@@ -2889,7 +2898,7 @@
           <t>רכישת דירה ברחוב הזיתים</t>
         </is>
       </c>
-      <c r="B9" s="3" t="n">
+      <c r="B9" s="9" t="n">
         <v>46128</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -2902,13 +2911,13 @@
           <t>סיכום פגישה</t>
         </is>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="E9" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="F9" s="5" t="n">
+      <c r="F9" s="11" t="n">
         <v>750</v>
       </c>
-      <c r="G9" s="5">
+      <c r="G9" s="11">
         <f>E9*F9</f>
         <v/>
       </c>
@@ -2919,7 +2928,7 @@
           <t>בקשה לצו מניעה</t>
         </is>
       </c>
-      <c r="B10" s="3" t="n">
+      <c r="B10" s="9" t="n">
         <v>46005</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -2932,13 +2941,13 @@
           <t>ניסוח מכתב התראה</t>
         </is>
       </c>
-      <c r="E10" s="4" t="n">
+      <c r="E10" s="10" t="n">
         <v>4.5</v>
       </c>
-      <c r="F10" s="5" t="n">
+      <c r="F10" s="11" t="n">
         <v>900</v>
       </c>
-      <c r="G10" s="5">
+      <c r="G10" s="11">
         <f>E10*F10</f>
         <v/>
       </c>
@@ -2949,7 +2958,7 @@
           <t>הסכם ממון - משפחת שרון</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n">
+      <c r="B11" s="9" t="n">
         <v>46020</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -2962,13 +2971,13 @@
           <t>בדיקת נסח טאבו</t>
         </is>
       </c>
-      <c r="E11" s="4" t="n">
+      <c r="E11" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="F11" s="5" t="n">
+      <c r="F11" s="11" t="n">
         <v>480</v>
       </c>
-      <c r="G11" s="5">
+      <c r="G11" s="11">
         <f>E11*F11</f>
         <v/>
       </c>
@@ -2979,7 +2988,7 @@
           <t>פלוני נ' חברת הבנייה</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n">
+      <c r="B12" s="9" t="n">
         <v>46022</v>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -2992,13 +3001,13 @@
           <t>הכנת תצהיר</t>
         </is>
       </c>
-      <c r="E12" s="4" t="n">
+      <c r="E12" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="F12" s="5" t="n">
+      <c r="F12" s="11" t="n">
         <v>650</v>
       </c>
-      <c r="G12" s="5">
+      <c r="G12" s="11">
         <f>E12*F12</f>
         <v/>
       </c>
@@ -3009,7 +3018,7 @@
           <t>עיזבון אלמוני</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>3.12.2025</t>
         </is>
@@ -3024,13 +3033,13 @@
           <t>דיון בבית המשפט</t>
         </is>
       </c>
-      <c r="E13" s="4" t="n">
+      <c r="E13" s="10" t="n">
         <v>1.5</v>
       </c>
-      <c r="F13" s="5" t="n">
+      <c r="F13" s="11" t="n">
         <v>750</v>
       </c>
-      <c r="G13" s="5">
+      <c r="G13" s="11">
         <f>E13*F13</f>
         <v/>
       </c>
@@ -3041,7 +3050,7 @@
           <t>רכישת דירה ברחוב הזיתים</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n">
+      <c r="B14" s="9" t="n">
         <v>46117</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -3054,13 +3063,13 @@
           <t>עיון בכתב ההגנה</t>
         </is>
       </c>
-      <c r="E14" s="4" t="n">
+      <c r="E14" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="F14" s="5" t="n">
+      <c r="F14" s="11" t="n">
         <v>900</v>
       </c>
-      <c r="G14" s="5">
+      <c r="G14" s="11">
         <f>E14*F14</f>
         <v/>
       </c>
@@ -3071,7 +3080,7 @@
           <t>בקשה לצו מניעה</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n">
+      <c r="B15" s="9" t="n">
         <v>46098</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -3084,13 +3093,13 @@
           <t>ישיבה עם הצד שכנגד</t>
         </is>
       </c>
-      <c r="E15" s="4" t="n">
+      <c r="E15" s="10" t="n">
         <v>2.5</v>
       </c>
-      <c r="F15" s="5" t="n">
+      <c r="F15" s="11" t="n">
         <v>480</v>
       </c>
-      <c r="G15" s="5">
+      <c r="G15" s="11">
         <f>E15*F15</f>
         <v/>
       </c>
@@ -3101,7 +3110,7 @@
           <t>הסכם ממון - משפחת שרון</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n">
+      <c r="B16" s="9" t="n">
         <v>45967</v>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -3114,13 +3123,13 @@
           <t>תיאום מול השמאי</t>
         </is>
       </c>
-      <c r="E16" s="4" t="n">
+      <c r="E16" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="F16" s="5" t="n">
+      <c r="F16" s="11" t="n">
         <v>650</v>
       </c>
-      <c r="G16" s="5">
+      <c r="G16" s="11">
         <f>E16*F16</f>
         <v/>
       </c>
@@ -3131,7 +3140,7 @@
           <t>פלוני נ' חברת הבנייה</t>
         </is>
       </c>
-      <c r="B17" s="3" t="n">
+      <c r="B17" s="9" t="n">
         <v>45965</v>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -3144,13 +3153,13 @@
           <t>מחקר פסיקה</t>
         </is>
       </c>
-      <c r="E17" s="4" t="n">
+      <c r="E17" s="10" t="n">
         <v>3.5</v>
       </c>
-      <c r="F17" s="5" t="n">
+      <c r="F17" s="11" t="n">
         <v>750</v>
       </c>
-      <c r="G17" s="5">
+      <c r="G17" s="11">
         <f>E17*F17</f>
         <v/>
       </c>
@@ -3161,7 +3170,7 @@
           <t>עיזבון אלמוני</t>
         </is>
       </c>
-      <c r="B18" s="3" t="n">
+      <c r="B18" s="9" t="n">
         <v>46037</v>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -3174,13 +3183,13 @@
           <t>עריכת טיוטת הסכם</t>
         </is>
       </c>
-      <c r="E18" s="4" t="n">
+      <c r="E18" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="F18" s="5" t="n">
+      <c r="F18" s="11" t="n">
         <v>900</v>
       </c>
-      <c r="G18" s="5">
+      <c r="G18" s="11">
         <f>E18*F18</f>
         <v/>
       </c>
@@ -3191,7 +3200,7 @@
           <t>רכישת דירה ברחוב הזיתים</t>
         </is>
       </c>
-      <c r="B19" s="3" t="n">
+      <c r="B19" s="9" t="n">
         <v>46086</v>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -3204,13 +3213,13 @@
           <t>שיחת ייעוץ עם הלקוח</t>
         </is>
       </c>
-      <c r="E19" s="4" t="n">
+      <c r="E19" s="10" t="n">
         <v>4.5</v>
       </c>
-      <c r="F19" s="5" t="n">
+      <c r="F19" s="11" t="n">
         <v>480</v>
       </c>
-      <c r="G19" s="5">
+      <c r="G19" s="11">
         <f>E19*F19</f>
         <v/>
       </c>
@@ -3221,7 +3230,7 @@
           <t>בקשה לצו מניעה</t>
         </is>
       </c>
-      <c r="B20" s="3" t="n">
+      <c r="B20" s="9" t="n">
         <v>46063</v>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -3234,13 +3243,13 @@
           <t>הכנה לדיון</t>
         </is>
       </c>
-      <c r="E20" s="4" t="n">
+      <c r="E20" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="F20" s="5" t="n">
+      <c r="F20" s="11" t="n">
         <v>650</v>
       </c>
-      <c r="G20" s="5">
+      <c r="G20" s="11">
         <f>E20*F20</f>
         <v/>
       </c>
@@ -3251,7 +3260,7 @@
           <t>הסכם ממון - משפחת שרון</t>
         </is>
       </c>
-      <c r="B21" s="3" t="n">
+      <c r="B21" s="9" t="n">
         <v>46002</v>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -3264,13 +3273,13 @@
           <t>סיכום פגישה</t>
         </is>
       </c>
-      <c r="E21" s="4" t="n">
+      <c r="E21" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="F21" s="5" t="n">
+      <c r="F21" s="11" t="n">
         <v>750</v>
       </c>
-      <c r="G21" s="5">
+      <c r="G21" s="11">
         <f>E21*F21</f>
         <v/>
       </c>
@@ -3281,7 +3290,7 @@
           <t>פלוני נ' חברת הבנייה</t>
         </is>
       </c>
-      <c r="B22" s="3" t="n">
+      <c r="B22" s="9" t="n">
         <v>45965</v>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -3294,13 +3303,13 @@
           <t>ניסוח מכתב התראה</t>
         </is>
       </c>
-      <c r="E22" s="4" t="n">
+      <c r="E22" s="10" t="n">
         <v>1.5</v>
       </c>
-      <c r="F22" s="5" t="n">
+      <c r="F22" s="11" t="n">
         <v>900</v>
       </c>
-      <c r="G22" s="5">
+      <c r="G22" s="11">
         <f>E22*F22</f>
         <v/>
       </c>
@@ -3311,7 +3320,7 @@
           <t>עיזבון אלמוני</t>
         </is>
       </c>
-      <c r="B23" s="3" t="n">
+      <c r="B23" s="9" t="n">
         <v>46059</v>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -3324,13 +3333,13 @@
           <t>בדיקת נסח טאבו</t>
         </is>
       </c>
-      <c r="E23" s="4" t="n">
+      <c r="E23" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="F23" s="5" t="n">
+      <c r="F23" s="11" t="n">
         <v>480</v>
       </c>
-      <c r="G23" s="5">
+      <c r="G23" s="11">
         <f>E23*F23</f>
         <v/>
       </c>
@@ -3341,7 +3350,7 @@
           <t>רכישת דירה ברחוב הזיתים</t>
         </is>
       </c>
-      <c r="B24" s="3" t="n">
+      <c r="B24" s="9" t="n">
         <v>45990</v>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -3354,13 +3363,13 @@
           <t>הכנת תצהיר</t>
         </is>
       </c>
-      <c r="E24" s="4" t="n">
+      <c r="E24" s="10" t="n">
         <v>2.5</v>
       </c>
-      <c r="F24" s="5" t="n">
+      <c r="F24" s="11" t="n">
         <v>820</v>
       </c>
-      <c r="G24" s="5">
+      <c r="G24" s="11">
         <f>E24*F24</f>
         <v/>
       </c>
@@ -3371,7 +3380,7 @@
           <t>בקשה לצו מניעה</t>
         </is>
       </c>
-      <c r="B25" s="3" t="n">
+      <c r="B25" s="9" t="n">
         <v>46117</v>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -3384,13 +3393,13 @@
           <t>דיון בבית המשפט</t>
         </is>
       </c>
-      <c r="E25" s="4" t="n">
+      <c r="E25" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="F25" s="5" t="n">
+      <c r="F25" s="11" t="n">
         <v>750</v>
       </c>
-      <c r="G25" s="5">
+      <c r="G25" s="11">
         <f>E25*F25</f>
         <v/>
       </c>
@@ -3401,7 +3410,7 @@
           <t>הסכם ממון - משפחת שרון</t>
         </is>
       </c>
-      <c r="B26" s="3" t="n">
+      <c r="B26" s="9" t="n">
         <v>46057</v>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -3414,13 +3423,13 @@
           <t>עיון בכתב ההגנה</t>
         </is>
       </c>
-      <c r="E26" s="4" t="n">
+      <c r="E26" s="10" t="n">
         <v>3.5</v>
       </c>
-      <c r="F26" s="5" t="n">
+      <c r="F26" s="11" t="n">
         <v>900</v>
       </c>
-      <c r="G26" s="5">
+      <c r="G26" s="11">
         <f>E26*F26</f>
         <v/>
       </c>
@@ -3431,7 +3440,7 @@
           <t>פלוני נ' חברת הבנייה</t>
         </is>
       </c>
-      <c r="B27" s="3" t="n">
+      <c r="B27" s="9" t="n">
         <v>46039</v>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -3444,13 +3453,13 @@
           <t>ישיבה עם הצד שכנגד</t>
         </is>
       </c>
-      <c r="E27" s="4" t="n">
+      <c r="E27" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="F27" s="5" t="n">
+      <c r="F27" s="11" t="n">
         <v>480</v>
       </c>
-      <c r="G27" s="5">
+      <c r="G27" s="11">
         <f>E27*F27</f>
         <v/>
       </c>
@@ -3461,7 +3470,7 @@
           <t>עיזבון אלמוני</t>
         </is>
       </c>
-      <c r="B28" s="3" t="n">
+      <c r="B28" s="9" t="n">
         <v>46128</v>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -3474,13 +3483,13 @@
           <t>תיאום מול השמאי</t>
         </is>
       </c>
-      <c r="E28" s="4" t="n">
+      <c r="E28" s="10" t="n">
         <v>4.5</v>
       </c>
-      <c r="F28" s="5" t="n">
+      <c r="F28" s="11" t="n">
         <v>650</v>
       </c>
-      <c r="G28" s="5">
+      <c r="G28" s="11">
         <f>E28*F28</f>
         <v/>
       </c>
@@ -3491,7 +3500,7 @@
           <t>רכישת דירה ברחוב הזיתים</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B29" s="9" t="inlineStr">
         <is>
           <t>2026-01-14</t>
         </is>
@@ -3506,13 +3515,13 @@
           <t>מחקר פסיקה</t>
         </is>
       </c>
-      <c r="E29" s="4" t="n">
+      <c r="E29" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="F29" s="5" t="n">
+      <c r="F29" s="11" t="n">
         <v>750</v>
       </c>
-      <c r="G29" s="5">
+      <c r="G29" s="11">
         <f>E29*F29</f>
         <v/>
       </c>
@@ -3523,7 +3532,7 @@
           <t>בקשה לצו מניעה</t>
         </is>
       </c>
-      <c r="B30" s="3" t="n">
+      <c r="B30" s="9" t="n">
         <v>46101</v>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -3536,13 +3545,13 @@
           <t>עריכת טיוטת הסכם</t>
         </is>
       </c>
-      <c r="E30" s="4" t="n">
+      <c r="E30" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="F30" s="5" t="n">
+      <c r="F30" s="11" t="n">
         <v>900</v>
       </c>
-      <c r="G30" s="5">
+      <c r="G30" s="11">
         <f>E30*F30</f>
         <v/>
       </c>
@@ -3553,7 +3562,7 @@
           <t>הסכם ממון - משפחת שרון</t>
         </is>
       </c>
-      <c r="B31" s="3" t="n">
+      <c r="B31" s="9" t="n">
         <v>46042</v>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -3566,13 +3575,13 @@
           <t>שיחת ייעוץ עם הלקוח</t>
         </is>
       </c>
-      <c r="E31" s="4" t="n">
+      <c r="E31" s="10" t="n">
         <v>1.5</v>
       </c>
-      <c r="F31" s="5" t="n">
+      <c r="F31" s="11" t="n">
         <v>480</v>
       </c>
-      <c r="G31" s="5">
+      <c r="G31" s="11">
         <f>E31*F31</f>
         <v/>
       </c>
@@ -3583,7 +3592,7 @@
           <t>פלוני נ' חברת הבנייה</t>
         </is>
       </c>
-      <c r="B32" s="3" t="n">
+      <c r="B32" s="9" t="n">
         <v>46036</v>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -3596,13 +3605,13 @@
           <t>הכנה לדיון</t>
         </is>
       </c>
-      <c r="E32" s="4" t="n">
+      <c r="E32" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="F32" s="5" t="n">
+      <c r="F32" s="11" t="n">
         <v>650</v>
       </c>
-      <c r="G32" s="5">
+      <c r="G32" s="11">
         <f>E32*F32</f>
         <v/>
       </c>
@@ -3613,7 +3622,7 @@
           <t>עיזבון אלמוני</t>
         </is>
       </c>
-      <c r="B33" s="3" t="n">
+      <c r="B33" s="9" t="n">
         <v>46030</v>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -3626,13 +3635,13 @@
           <t>סיכום פגישה</t>
         </is>
       </c>
-      <c r="E33" s="4" t="n">
+      <c r="E33" s="10" t="n">
         <v>2.5</v>
       </c>
-      <c r="F33" s="5" t="n">
+      <c r="F33" s="11" t="n">
         <v>750</v>
       </c>
-      <c r="G33" s="5">
+      <c r="G33" s="11">
         <f>E33*F33</f>
         <v/>
       </c>
@@ -3643,7 +3652,7 @@
           <t>רכישת דירה ברחוב הזיתים</t>
         </is>
       </c>
-      <c r="B34" s="3" t="n">
+      <c r="B34" s="9" t="n">
         <v>46103</v>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -3656,13 +3665,13 @@
           <t>ניסוח מכתב התראה</t>
         </is>
       </c>
-      <c r="E34" s="4" t="n">
+      <c r="E34" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="F34" s="5" t="n">
+      <c r="F34" s="11" t="n">
         <v>900</v>
       </c>
-      <c r="G34" s="5">
+      <c r="G34" s="11">
         <f>E34*F34</f>
         <v/>
       </c>
@@ -3673,7 +3682,7 @@
           <t>בקשה לצו מניעה</t>
         </is>
       </c>
-      <c r="B35" s="3" t="n">
+      <c r="B35" s="9" t="n">
         <v>45987</v>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -3686,15 +3695,15 @@
           <t>בדיקת נסח טאבו</t>
         </is>
       </c>
-      <c r="E35" s="4" t="inlineStr">
+      <c r="E35" s="10" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F35" s="5" t="n">
+      <c r="F35" s="11" t="n">
         <v>480</v>
       </c>
-      <c r="G35" s="5">
+      <c r="G35" s="11">
         <f>E35*F35</f>
         <v/>
       </c>
@@ -3705,7 +3714,7 @@
           <t>הסכם ממון - משפחת שרון</t>
         </is>
       </c>
-      <c r="B36" s="3" t="n">
+      <c r="B36" s="9" t="n">
         <v>46105</v>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -3718,13 +3727,13 @@
           <t>הכנת תצהיר</t>
         </is>
       </c>
-      <c r="E36" s="4" t="n">
+      <c r="E36" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="F36" s="5" t="n">
+      <c r="F36" s="11" t="n">
         <v>650</v>
       </c>
-      <c r="G36" s="5">
+      <c r="G36" s="11">
         <f>E36*F36</f>
         <v/>
       </c>
@@ -3735,7 +3744,7 @@
           <t>פלוני נ' חברת הבנייה</t>
         </is>
       </c>
-      <c r="B37" s="3" t="n">
+      <c r="B37" s="9" t="n">
         <v>46088</v>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -3748,13 +3757,13 @@
           <t>דיון בבית המשפט</t>
         </is>
       </c>
-      <c r="E37" s="4" t="n">
+      <c r="E37" s="10" t="n">
         <v>4.5</v>
       </c>
-      <c r="F37" s="5" t="n">
+      <c r="F37" s="11" t="n">
         <v>750</v>
       </c>
-      <c r="G37" s="5">
+      <c r="G37" s="11">
         <f>E37*F37</f>
         <v/>
       </c>
@@ -3765,7 +3774,7 @@
           <t>עיזבון אלמוני</t>
         </is>
       </c>
-      <c r="B38" s="3" t="n">
+      <c r="B38" s="9" t="n">
         <v>46071</v>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -3778,13 +3787,13 @@
           <t>עיון בכתב ההגנה</t>
         </is>
       </c>
-      <c r="E38" s="4" t="n">
+      <c r="E38" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="F38" s="5" t="n">
+      <c r="F38" s="11" t="n">
         <v>900</v>
       </c>
-      <c r="G38" s="5">
+      <c r="G38" s="11">
         <f>E38*F38</f>
         <v/>
       </c>
@@ -3795,7 +3804,7 @@
           <t>רכישת דירה ברחוב הזיתים</t>
         </is>
       </c>
-      <c r="B39" s="3" t="n">
+      <c r="B39" s="9" t="n">
         <v>45981</v>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -3808,13 +3817,13 @@
           <t>ישיבה עם הצד שכנגד</t>
         </is>
       </c>
-      <c r="E39" s="4" t="n">
+      <c r="E39" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="F39" s="5" t="n">
+      <c r="F39" s="11" t="n">
         <v>480</v>
       </c>
-      <c r="G39" s="5">
+      <c r="G39" s="11">
         <f>E39*F39</f>
         <v/>
       </c>
@@ -3825,7 +3834,7 @@
           <t>בקשה לצו מניעה</t>
         </is>
       </c>
-      <c r="B40" s="3" t="n">
+      <c r="B40" s="9" t="n">
         <v>46016</v>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -3838,13 +3847,13 @@
           <t>תיאום מול השמאי</t>
         </is>
       </c>
-      <c r="E40" s="4" t="n">
+      <c r="E40" s="10" t="n">
         <v>1.5</v>
       </c>
-      <c r="F40" s="5" t="n">
+      <c r="F40" s="11" t="n">
         <v>650</v>
       </c>
-      <c r="G40" s="5">
+      <c r="G40" s="11">
         <f>E40*F40</f>
         <v/>
       </c>
@@ -3855,7 +3864,7 @@
           <t>הסכם ממון - משפחת שרון</t>
         </is>
       </c>
-      <c r="B41" s="3" t="n">
+      <c r="B41" s="9" t="n">
         <v>46119</v>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -3868,13 +3877,13 @@
           <t>מחקר פסיקה</t>
         </is>
       </c>
-      <c r="E41" s="4" t="n">
+      <c r="E41" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="F41" s="5" t="n">
+      <c r="F41" s="11" t="n">
         <v>750</v>
       </c>
-      <c r="G41" s="5">
+      <c r="G41" s="11">
         <f>E41*F41</f>
         <v/>
       </c>
@@ -3885,7 +3894,7 @@
           <t>פלוני נ' חברת הבנייה</t>
         </is>
       </c>
-      <c r="B42" s="3" t="n">
+      <c r="B42" s="9" t="n">
         <v>46068</v>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -3898,13 +3907,13 @@
           <t>עריכת טיוטת הסכם</t>
         </is>
       </c>
-      <c r="E42" s="4" t="n">
+      <c r="E42" s="10" t="n">
         <v>2.5</v>
       </c>
-      <c r="F42" s="5" t="n">
+      <c r="F42" s="11" t="n">
         <v>900</v>
       </c>
-      <c r="G42" s="5">
+      <c r="G42" s="11">
         <f>E42*F42</f>
         <v/>
       </c>
@@ -3915,7 +3924,7 @@
           <t>עיזבון אלמוני</t>
         </is>
       </c>
-      <c r="B43" s="3" t="n">
+      <c r="B43" s="9" t="n">
         <v>46034</v>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -3928,11 +3937,11 @@
           <t>שיחת ייעוץ עם הלקוח</t>
         </is>
       </c>
-      <c r="E43" s="4" t="n">
+      <c r="E43" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="F43" s="5" t="n"/>
-      <c r="G43" s="5">
+      <c r="F43" s="11" t="n"/>
+      <c r="G43" s="11">
         <f>E43*F43</f>
         <v/>
       </c>
@@ -3943,7 +3952,7 @@
           <t>רכישת דירה ברחוב הזיתים</t>
         </is>
       </c>
-      <c r="B44" s="3" t="n">
+      <c r="B44" s="9" t="n">
         <v>45968</v>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -3956,13 +3965,13 @@
           <t>הכנה לדיון</t>
         </is>
       </c>
-      <c r="E44" s="4" t="n">
+      <c r="E44" s="10" t="n">
         <v>3.5</v>
       </c>
-      <c r="F44" s="5" t="n">
+      <c r="F44" s="11" t="n">
         <v>650</v>
       </c>
-      <c r="G44" s="5">
+      <c r="G44" s="11">
         <f>E44*F44</f>
         <v/>
       </c>
@@ -3973,7 +3982,7 @@
           <t>בקשה לצו מניעה</t>
         </is>
       </c>
-      <c r="B45" s="3" t="n">
+      <c r="B45" s="9" t="n">
         <v>46113</v>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -3986,13 +3995,13 @@
           <t>סיכום פגישה</t>
         </is>
       </c>
-      <c r="E45" s="4" t="n">
+      <c r="E45" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="F45" s="5" t="n">
+      <c r="F45" s="11" t="n">
         <v>750</v>
       </c>
-      <c r="G45" s="5">
+      <c r="G45" s="11">
         <f>E45*F45</f>
         <v/>
       </c>
@@ -4003,7 +4012,7 @@
           <t>הסכם ממון - משפחת שרון</t>
         </is>
       </c>
-      <c r="B46" s="3" t="n">
+      <c r="B46" s="9" t="n">
         <v>45989</v>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -4016,13 +4025,13 @@
           <t>ניסוח מכתב התראה</t>
         </is>
       </c>
-      <c r="E46" s="4" t="n">
+      <c r="E46" s="10" t="n">
         <v>4.5</v>
       </c>
-      <c r="F46" s="5" t="n">
+      <c r="F46" s="11" t="n">
         <v>900</v>
       </c>
-      <c r="G46" s="5">
+      <c r="G46" s="11">
         <f>E46*F46</f>
         <v/>
       </c>
@@ -4033,7 +4042,7 @@
           <t>הסכם ממון - משפחת שרון</t>
         </is>
       </c>
-      <c r="B47" s="3" t="n">
+      <c r="B47" s="9" t="n">
         <v>45989</v>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -4046,13 +4055,13 @@
           <t>ניסוח מכתב התראה</t>
         </is>
       </c>
-      <c r="E47" s="4" t="n">
+      <c r="E47" s="10" t="n">
         <v>4.5</v>
       </c>
-      <c r="F47" s="5" t="n">
+      <c r="F47" s="11" t="n">
         <v>900</v>
       </c>
-      <c r="G47" s="5">
+      <c r="G47" s="11">
         <f>E47*F47</f>
         <v/>
       </c>
@@ -4063,7 +4072,7 @@
           <t>פלוני נ' חברת הבנייה</t>
         </is>
       </c>
-      <c r="B48" s="3" t="n">
+      <c r="B48" s="9" t="n">
         <v>46045</v>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -4076,13 +4085,13 @@
           <t>בדיקת נסח טאבו</t>
         </is>
       </c>
-      <c r="E48" s="4" t="n">
+      <c r="E48" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="F48" s="5" t="n">
+      <c r="F48" s="11" t="n">
         <v>480</v>
       </c>
-      <c r="G48" s="5">
+      <c r="G48" s="11">
         <f>E48*F48</f>
         <v/>
       </c>
@@ -4093,7 +4102,7 @@
           <t>עיזבון אלמוני</t>
         </is>
       </c>
-      <c r="B49" s="3" t="n">
+      <c r="B49" s="9" t="n">
         <v>46033</v>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -4106,13 +4115,13 @@
           <t>הכנת תצהיר</t>
         </is>
       </c>
-      <c r="E49" s="4" t="n">
+      <c r="E49" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="F49" s="5" t="n">
+      <c r="F49" s="11" t="n">
         <v>650</v>
       </c>
-      <c r="G49" s="5">
+      <c r="G49" s="11">
         <f>E49*F49</f>
         <v/>
       </c>
@@ -4123,7 +4132,7 @@
           <t>רכישת דירה ברחוב הזיתים</t>
         </is>
       </c>
-      <c r="B50" s="3" t="n">
+      <c r="B50" s="9" t="n">
         <v>46000</v>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -4136,13 +4145,13 @@
           <t>דיון בבית המשפט</t>
         </is>
       </c>
-      <c r="E50" s="4" t="n">
+      <c r="E50" s="10" t="n">
         <v>1.5</v>
       </c>
-      <c r="F50" s="5" t="n">
+      <c r="F50" s="11" t="n">
         <v>750</v>
       </c>
-      <c r="G50" s="5">
+      <c r="G50" s="11">
         <f>E50*F50</f>
         <v/>
       </c>
@@ -4153,7 +4162,7 @@
           <t>בקשה לצו מניעה</t>
         </is>
       </c>
-      <c r="B51" s="3" t="n">
+      <c r="B51" s="9" t="n">
         <v>45992</v>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -4166,13 +4175,13 @@
           <t>עיון בכתב ההגנה</t>
         </is>
       </c>
-      <c r="E51" s="4" t="n">
+      <c r="E51" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="F51" s="5" t="n">
+      <c r="F51" s="11" t="n">
         <v>900</v>
       </c>
-      <c r="G51" s="5">
+      <c r="G51" s="11">
         <f>E51*F51</f>
         <v/>
       </c>
@@ -4183,7 +4192,7 @@
           <t>פלוני נ' חברת הבנייה</t>
         </is>
       </c>
-      <c r="B52" s="3" t="n">
+      <c r="B52" s="9" t="n">
         <v>46010</v>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -4196,13 +4205,13 @@
           <t>תיאום מול השמאי</t>
         </is>
       </c>
-      <c r="E52" s="4" t="n">
+      <c r="E52" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="F52" s="5" t="n">
+      <c r="F52" s="11" t="n">
         <v>650</v>
       </c>
-      <c r="G52" s="5">
+      <c r="G52" s="11">
         <f>E52*F52</f>
         <v/>
       </c>
@@ -4213,7 +4222,7 @@
           <t>עיזבון אלמוני</t>
         </is>
       </c>
-      <c r="B53" s="3" t="n">
+      <c r="B53" s="9" t="n">
         <v>46102</v>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -4226,13 +4235,13 @@
           <t>מחקר פסיקה</t>
         </is>
       </c>
-      <c r="E53" s="4" t="n">
+      <c r="E53" s="10" t="n">
         <v>3.5</v>
       </c>
-      <c r="F53" s="5" t="n">
+      <c r="F53" s="11" t="n">
         <v>750</v>
       </c>
-      <c r="G53" s="5">
+      <c r="G53" s="11">
         <f>E53*F53</f>
         <v/>
       </c>
@@ -4243,7 +4252,7 @@
           <t>רכישת דירה ברחוב הזיתים</t>
         </is>
       </c>
-      <c r="B54" s="3" t="n">
+      <c r="B54" s="9" t="n">
         <v>46004</v>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -4256,13 +4265,13 @@
           <t>עריכת טיוטת הסכם</t>
         </is>
       </c>
-      <c r="E54" s="4" t="n">
+      <c r="E54" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="F54" s="5" t="n">
+      <c r="F54" s="11" t="n">
         <v>900</v>
       </c>
-      <c r="G54" s="5">
+      <c r="G54" s="11">
         <f>E54*F54</f>
         <v/>
       </c>
@@ -4273,7 +4282,7 @@
           <t>בקשה לצו מניעה</t>
         </is>
       </c>
-      <c r="B55" s="3" t="n">
+      <c r="B55" s="9" t="n">
         <v>46063</v>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -4286,13 +4295,13 @@
           <t>שיחת ייעוץ עם הלקוח</t>
         </is>
       </c>
-      <c r="E55" s="4" t="n">
+      <c r="E55" s="10" t="n">
         <v>4.5</v>
       </c>
-      <c r="F55" s="5" t="n">
+      <c r="F55" s="11" t="n">
         <v>480</v>
       </c>
-      <c r="G55" s="5">
+      <c r="G55" s="11">
         <f>E55*F55</f>
         <v/>
       </c>
@@ -4303,7 +4312,7 @@
           <t>הסכם ממון - משפחת שרון</t>
         </is>
       </c>
-      <c r="B56" s="3" t="n">
+      <c r="B56" s="9" t="n">
         <v>46066</v>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -4316,13 +4325,13 @@
           <t>הכנה לדיון</t>
         </is>
       </c>
-      <c r="E56" s="4" t="n">
+      <c r="E56" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="F56" s="5" t="n">
+      <c r="F56" s="11" t="n">
         <v>650</v>
       </c>
-      <c r="G56" s="5">
+      <c r="G56" s="11">
         <f>E56*F56</f>
         <v/>
       </c>
@@ -4333,7 +4342,7 @@
           <t>פלוני נ' חברת הבנייה</t>
         </is>
       </c>
-      <c r="B57" s="3" t="n">
+      <c r="B57" s="9" t="n">
         <v>46113</v>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -4346,13 +4355,13 @@
           <t>סיכום פגישה</t>
         </is>
       </c>
-      <c r="E57" s="4" t="n">
+      <c r="E57" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="F57" s="5" t="n">
+      <c r="F57" s="11" t="n">
         <v>750</v>
       </c>
-      <c r="G57" s="5">
+      <c r="G57" s="11">
         <f>E57*F57</f>
         <v/>
       </c>
@@ -4363,7 +4372,7 @@
           <t>עיזבון אלמוני</t>
         </is>
       </c>
-      <c r="B58" s="3" t="n">
+      <c r="B58" s="9" t="n">
         <v>46073</v>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -4376,13 +4385,13 @@
           <t>ניסוח מכתב התראה</t>
         </is>
       </c>
-      <c r="E58" s="4" t="n">
+      <c r="E58" s="10" t="n">
         <v>1.5</v>
       </c>
-      <c r="F58" s="5" t="n">
+      <c r="F58" s="11" t="n">
         <v>900</v>
       </c>
-      <c r="G58" s="5">
+      <c r="G58" s="11">
         <f>E58*F58</f>
         <v/>
       </c>
@@ -4393,7 +4402,7 @@
           <t>רכישת דירה ברחוב הזיתים</t>
         </is>
       </c>
-      <c r="B59" s="3" t="n">
+      <c r="B59" s="9" t="n">
         <v>46020</v>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -4406,13 +4415,13 @@
           <t>בדיקת נסח טאבו</t>
         </is>
       </c>
-      <c r="E59" s="4" t="n">
+      <c r="E59" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="F59" s="5" t="n">
+      <c r="F59" s="11" t="n">
         <v>480</v>
       </c>
-      <c r="G59" s="5">
+      <c r="G59" s="11">
         <f>E59*F59</f>
         <v/>
       </c>
@@ -4470,10 +4479,10 @@
           <t>שותפה</t>
         </is>
       </c>
-      <c r="C2" s="5" t="n">
+      <c r="C2" s="11" t="n">
         <v>900</v>
       </c>
-      <c r="D2" s="3" t="n">
+      <c r="D2" s="9" t="n">
         <v>45658</v>
       </c>
     </row>
@@ -4488,10 +4497,10 @@
           <t>עורך דין בכיר</t>
         </is>
       </c>
-      <c r="C3" s="5" t="n">
+      <c r="C3" s="11" t="n">
         <v>750</v>
       </c>
-      <c r="D3" s="3" t="n">
+      <c r="D3" s="9" t="n">
         <v>45658</v>
       </c>
     </row>
@@ -4506,10 +4515,10 @@
           <t>עורכת דין</t>
         </is>
       </c>
-      <c r="C4" s="5" t="n">
+      <c r="C4" s="11" t="n">
         <v>650</v>
       </c>
-      <c r="D4" s="3" t="n">
+      <c r="D4" s="9" t="n">
         <v>45839</v>
       </c>
     </row>
@@ -4524,10 +4533,10 @@
           <t>מתמחה</t>
         </is>
       </c>
-      <c r="C5" s="5" t="n">
+      <c r="C5" s="11" t="n">
         <v>480</v>
       </c>
-      <c r="D5" s="3" t="n">
+      <c r="D5" s="9" t="n">
         <v>45901</v>
       </c>
     </row>
@@ -4586,7 +4595,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="n">
+      <c r="A2" s="9" t="n">
         <v>45728</v>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -4610,7 +4619,7 @@
       <c r="F2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="n">
+      <c r="A3" s="9" t="n">
         <v>45781</v>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -4634,7 +4643,7 @@
       <c r="F3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>18.6.2025</t>
         </is>
@@ -4657,14 +4666,10 @@
       <c r="E4" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>תאריך כטקסט</t>
-        </is>
-      </c>
+      <c r="F4" s="2" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n">
+      <c r="A5" s="9" t="n">
         <v>45826</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -4685,14 +4690,10 @@
       <c r="E5" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>אותו אירוע פעמיים</t>
-        </is>
-      </c>
+      <c r="F5" s="2" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="n">
+      <c r="A6" s="9" t="n">
         <v>45890</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -4714,7 +4715,7 @@
       <c r="F6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="n">
+      <c r="A7" s="9" t="n">
         <v>45902</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -4738,7 +4739,7 @@
       <c r="F7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>2025-10-30</t>
         </is>
@@ -4761,14 +4762,10 @@
       <c r="E8" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>תאריך כטקסט</t>
-        </is>
-      </c>
+      <c r="F8" s="2" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="n"/>
+      <c r="A9" s="9" t="n"/>
       <c r="B9" s="2" t="inlineStr">
         <is>
           <t>התקבלה תשובת חברת הבנייה</t>
@@ -4787,14 +4784,10 @@
       <c r="E9" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>אין תאריך במסמך</t>
-        </is>
-      </c>
+      <c r="F9" s="2" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="n">
+      <c r="A10" s="9" t="n">
         <v>46030</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -4818,7 +4811,7 @@
       <c r="F10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="n">
+      <c r="A11" s="9" t="n">
         <v>46072</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -4912,7 +4905,7 @@
           <t>הסכם בנייה</t>
         </is>
       </c>
-      <c r="C2" s="3" t="n">
+      <c r="C2" s="9" t="n">
         <v>45728</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -4945,7 +4938,7 @@
           <t>היתר בנייה</t>
         </is>
       </c>
-      <c r="C3" s="3" t="n">
+      <c r="C3" s="9" t="n">
         <v>45781</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -4978,7 +4971,7 @@
           <t>מכתב עיכוב מסירה</t>
         </is>
       </c>
-      <c r="C4" s="3" t="n">
+      <c r="C4" s="9" t="n">
         <v>45826</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -5011,7 +5004,7 @@
           <t>אישור תשלום רביעי</t>
         </is>
       </c>
-      <c r="C5" s="3" t="n">
+      <c r="C5" s="9" t="n">
         <v>45890</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -5044,7 +5037,7 @@
           <t>פרוטוקול סיור באתר</t>
         </is>
       </c>
-      <c r="C6" s="3" t="n">
+      <c r="C6" s="9" t="n">
         <v>45902</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -5077,7 +5070,7 @@
           <t>מכתב התראה</t>
         </is>
       </c>
-      <c r="C7" s="3" t="n">
+      <c r="C7" s="9" t="n">
         <v>45960</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -5110,7 +5103,7 @@
           <t>תשובת חברת הבנייה</t>
         </is>
       </c>
-      <c r="C8" s="3" t="n">
+      <c r="C8" s="9" t="n">
         <v>45985</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -5143,7 +5136,7 @@
           <t>חוות דעת מהנדס</t>
         </is>
       </c>
-      <c r="C9" s="3" t="n">
+      <c r="C9" s="9" t="n">
         <v>46006</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -5226,7 +5219,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="n">
+      <c r="A2" s="9" t="n">
         <v>45903</v>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -5239,17 +5232,17 @@
           <t>100000</t>
         </is>
       </c>
-      <c r="D2" s="5" t="n"/>
-      <c r="E2" s="5" t="n">
+      <c r="D2" s="11" t="n"/>
+      <c r="E2" s="11" t="n">
         <v>21500</v>
       </c>
-      <c r="F2" s="5" t="n">
+      <c r="F2" s="11" t="n">
         <v>105500</v>
       </c>
       <c r="G2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="n">
+      <c r="A3" s="9" t="n">
         <v>45906</v>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -5262,17 +5255,17 @@
           <t>100007</t>
         </is>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="D3" s="11" t="n">
         <v>4037</v>
       </c>
-      <c r="E3" s="5" t="n"/>
-      <c r="F3" s="5" t="n">
+      <c r="E3" s="11" t="n"/>
+      <c r="F3" s="11" t="n">
         <v>101463</v>
       </c>
       <c r="G3" s="2" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n">
+      <c r="A4" s="9" t="n">
         <v>45910</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -5285,17 +5278,17 @@
           <t>100014</t>
         </is>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="D4" s="11" t="n">
         <v>3894</v>
       </c>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="5" t="n">
+      <c r="E4" s="11" t="n"/>
+      <c r="F4" s="11" t="n">
         <v>97569</v>
       </c>
       <c r="G4" s="2" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n">
+      <c r="A5" s="9" t="n">
         <v>45915</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -5308,17 +5301,17 @@
           <t>100021</t>
         </is>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="D5" s="11" t="n">
         <v>6561</v>
       </c>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="n">
+      <c r="E5" s="11" t="n"/>
+      <c r="F5" s="11" t="n">
         <v>91008</v>
       </c>
       <c r="G5" s="2" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="n">
+      <c r="A6" s="9" t="n">
         <v>45917</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -5331,19 +5324,19 @@
           <t>100028</t>
         </is>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="D6" s="11" t="n">
         <v>148</v>
       </c>
-      <c r="E6" s="5" t="n">
+      <c r="E6" s="11" t="n">
         <v>835</v>
       </c>
-      <c r="F6" s="5" t="n">
+      <c r="F6" s="11" t="n">
         <v>91695</v>
       </c>
       <c r="G6" s="2" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="n">
+      <c r="A7" s="9" t="n">
         <v>45920</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -5356,17 +5349,17 @@
           <t>100035</t>
         </is>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="D7" s="11" t="n">
         <v>2300</v>
       </c>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7" s="5" t="n">
+      <c r="E7" s="11" t="n"/>
+      <c r="F7" s="11" t="n">
         <v>89395</v>
       </c>
       <c r="G7" s="2" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="n">
+      <c r="A8" s="9" t="n">
         <v>45924</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -5379,17 +5372,17 @@
           <t>100042</t>
         </is>
       </c>
-      <c r="D8" s="5" t="n">
+      <c r="D8" s="11" t="n">
         <v>1277</v>
       </c>
-      <c r="E8" s="5" t="n"/>
-      <c r="F8" s="5" t="n">
+      <c r="E8" s="11" t="n"/>
+      <c r="F8" s="11" t="n">
         <v>88118</v>
       </c>
       <c r="G8" s="2" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="n">
+      <c r="A9" s="9" t="n">
         <v>45929</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -5402,17 +5395,17 @@
           <t>100049</t>
         </is>
       </c>
-      <c r="D9" s="5" t="n">
+      <c r="D9" s="11" t="n">
         <v>5074</v>
       </c>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="5" t="n">
+      <c r="E9" s="11" t="n"/>
+      <c r="F9" s="11" t="n">
         <v>83044</v>
       </c>
       <c r="G9" s="2" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="n">
+      <c r="A10" s="9" t="n">
         <v>45931</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -5425,17 +5418,17 @@
           <t>100056</t>
         </is>
       </c>
-      <c r="D10" s="5" t="n">
+      <c r="D10" s="11" t="n">
         <v>751</v>
       </c>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n">
+      <c r="E10" s="11" t="n"/>
+      <c r="F10" s="11" t="n">
         <v>82293</v>
       </c>
       <c r="G10" s="2" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="n">
+      <c r="A11" s="9" t="n">
         <v>45934</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -5448,17 +5441,17 @@
           <t>100063</t>
         </is>
       </c>
-      <c r="D11" s="5" t="n">
+      <c r="D11" s="11" t="n">
         <v>2148</v>
       </c>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="5" t="n">
+      <c r="E11" s="11" t="n"/>
+      <c r="F11" s="11" t="n">
         <v>80145</v>
       </c>
       <c r="G11" s="2" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="n">
+      <c r="A12" s="9" t="n">
         <v>45938</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -5471,17 +5464,17 @@
           <t>100070</t>
         </is>
       </c>
-      <c r="D12" s="5" t="n">
+      <c r="D12" s="11" t="n">
         <v>8900</v>
       </c>
-      <c r="E12" s="5" t="n"/>
-      <c r="F12" s="5" t="n">
+      <c r="E12" s="11" t="n"/>
+      <c r="F12" s="11" t="n">
         <v>71245</v>
       </c>
       <c r="G12" s="2" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="n">
+      <c r="A13" s="9" t="n">
         <v>45943</v>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -5494,19 +5487,19 @@
           <t>100077</t>
         </is>
       </c>
-      <c r="D13" s="5" t="n">
+      <c r="D13" s="11" t="n">
         <v>37</v>
       </c>
-      <c r="E13" s="5" t="n">
+      <c r="E13" s="11" t="n">
         <v>122</v>
       </c>
-      <c r="F13" s="5" t="n">
+      <c r="F13" s="11" t="n">
         <v>71330</v>
       </c>
       <c r="G13" s="2" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="n">
+      <c r="A14" s="9" t="n">
         <v>45945</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -5519,19 +5512,19 @@
           <t>100084</t>
         </is>
       </c>
-      <c r="D14" s="5" t="n">
+      <c r="D14" s="11" t="n">
         <v>74</v>
       </c>
-      <c r="E14" s="5" t="n">
+      <c r="E14" s="11" t="n">
         <v>21500</v>
       </c>
-      <c r="F14" s="5" t="n">
+      <c r="F14" s="11" t="n">
         <v>92756</v>
       </c>
       <c r="G14" s="2" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="n">
+      <c r="A15" s="9" t="n">
         <v>45948</v>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -5544,17 +5537,17 @@
           <t>100091</t>
         </is>
       </c>
-      <c r="D15" s="5" t="n">
+      <c r="D15" s="11" t="n">
         <v>4111</v>
       </c>
-      <c r="E15" s="5" t="n"/>
-      <c r="F15" s="5" t="n">
+      <c r="E15" s="11" t="n"/>
+      <c r="F15" s="11" t="n">
         <v>88645</v>
       </c>
       <c r="G15" s="2" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="n">
+      <c r="A16" s="9" t="n">
         <v>45952</v>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -5567,17 +5560,17 @@
           <t>100098</t>
         </is>
       </c>
-      <c r="D16" s="5" t="n">
+      <c r="D16" s="11" t="n">
         <v>3968</v>
       </c>
-      <c r="E16" s="5" t="n"/>
-      <c r="F16" s="5" t="n">
+      <c r="E16" s="11" t="n"/>
+      <c r="F16" s="11" t="n">
         <v>84677</v>
       </c>
       <c r="G16" s="2" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="n">
+      <c r="A17" s="9" t="n">
         <v>45957</v>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -5590,17 +5583,17 @@
           <t>100105</t>
         </is>
       </c>
-      <c r="D17" s="5" t="n">
+      <c r="D17" s="11" t="n">
         <v>6450</v>
       </c>
-      <c r="E17" s="5" t="n"/>
-      <c r="F17" s="5" t="n">
+      <c r="E17" s="11" t="n"/>
+      <c r="F17" s="11" t="n">
         <v>78227</v>
       </c>
       <c r="G17" s="2" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="n">
+      <c r="A18" s="9" t="n">
         <v>45959</v>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -5613,19 +5606,19 @@
           <t>100112</t>
         </is>
       </c>
-      <c r="D18" s="5" t="n">
+      <c r="D18" s="11" t="n">
         <v>37</v>
       </c>
-      <c r="E18" s="5" t="n">
+      <c r="E18" s="11" t="n">
         <v>835</v>
       </c>
-      <c r="F18" s="5" t="n">
+      <c r="F18" s="11" t="n">
         <v>79025</v>
       </c>
       <c r="G18" s="2" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="n">
+      <c r="A19" s="9" t="n">
         <v>45962</v>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -5638,17 +5631,17 @@
           <t>100119</t>
         </is>
       </c>
-      <c r="D19" s="5" t="n">
+      <c r="D19" s="11" t="n">
         <v>2374</v>
       </c>
-      <c r="E19" s="5" t="n"/>
-      <c r="F19" s="5" t="n">
+      <c r="E19" s="11" t="n"/>
+      <c r="F19" s="11" t="n">
         <v>76651</v>
       </c>
       <c r="G19" s="2" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="n">
+      <c r="A20" s="9" t="n">
         <v>45966</v>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -5661,17 +5654,17 @@
           <t>100126</t>
         </is>
       </c>
-      <c r="D20" s="5" t="n">
+      <c r="D20" s="11" t="n">
         <v>1351</v>
       </c>
-      <c r="E20" s="5" t="n"/>
-      <c r="F20" s="5" t="n">
+      <c r="E20" s="11" t="n"/>
+      <c r="F20" s="11" t="n">
         <v>75300</v>
       </c>
       <c r="G20" s="2" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="n">
+      <c r="A21" s="9" t="n">
         <v>45971</v>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -5684,17 +5677,17 @@
           <t>100133</t>
         </is>
       </c>
-      <c r="D21" s="5" t="n">
+      <c r="D21" s="11" t="n">
         <v>5148</v>
       </c>
-      <c r="E21" s="5" t="n"/>
-      <c r="F21" s="5" t="n">
+      <c r="E21" s="11" t="n"/>
+      <c r="F21" s="11" t="n">
         <v>70152</v>
       </c>
       <c r="G21" s="2" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="n">
+      <c r="A22" s="9" t="n">
         <v>45973</v>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -5707,17 +5700,17 @@
           <t>100140</t>
         </is>
       </c>
-      <c r="D22" s="5" t="n">
+      <c r="D22" s="11" t="n">
         <v>640</v>
       </c>
-      <c r="E22" s="5" t="n"/>
-      <c r="F22" s="5" t="n">
+      <c r="E22" s="11" t="n"/>
+      <c r="F22" s="11" t="n">
         <v>69512</v>
       </c>
       <c r="G22" s="2" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="n">
+      <c r="A23" s="9" t="n">
         <v>45976</v>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -5730,17 +5723,17 @@
           <t>100147</t>
         </is>
       </c>
-      <c r="D23" s="5" t="n">
+      <c r="D23" s="11" t="n">
         <v>2037</v>
       </c>
-      <c r="E23" s="5" t="n"/>
-      <c r="F23" s="5" t="n">
+      <c r="E23" s="11" t="n"/>
+      <c r="F23" s="11" t="n">
         <v>67475</v>
       </c>
       <c r="G23" s="2" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="n">
+      <c r="A24" s="9" t="n">
         <v>45980</v>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -5753,17 +5746,17 @@
           <t>100154</t>
         </is>
       </c>
-      <c r="D24" s="5" t="n">
+      <c r="D24" s="11" t="n">
         <v>8974</v>
       </c>
-      <c r="E24" s="5" t="n"/>
-      <c r="F24" s="5" t="n">
+      <c r="E24" s="11" t="n"/>
+      <c r="F24" s="11" t="n">
         <v>58501</v>
       </c>
       <c r="G24" s="2" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="n">
+      <c r="A25" s="9" t="n">
         <v>45985</v>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -5776,19 +5769,19 @@
           <t>100161</t>
         </is>
       </c>
-      <c r="D25" s="5" t="n">
+      <c r="D25" s="11" t="n">
         <v>111</v>
       </c>
-      <c r="E25" s="5" t="n">
+      <c r="E25" s="11" t="n">
         <v>122</v>
       </c>
-      <c r="F25" s="5" t="n">
+      <c r="F25" s="11" t="n">
         <v>58512</v>
       </c>
       <c r="G25" s="2" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="n">
+      <c r="A26" s="9" t="n">
         <v>45987</v>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -5801,19 +5794,19 @@
           <t>100168</t>
         </is>
       </c>
-      <c r="D26" s="5" t="n">
+      <c r="D26" s="11" t="n">
         <v>148</v>
       </c>
-      <c r="E26" s="5" t="n">
+      <c r="E26" s="11" t="n">
         <v>21500</v>
       </c>
-      <c r="F26" s="5" t="n">
+      <c r="F26" s="11" t="n">
         <v>79864</v>
       </c>
       <c r="G26" s="2" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="n">
+      <c r="A27" s="9" t="n">
         <v>45990</v>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -5826,17 +5819,17 @@
           <t>100175</t>
         </is>
       </c>
-      <c r="D27" s="5" t="n">
+      <c r="D27" s="11" t="n">
         <v>4000</v>
       </c>
-      <c r="E27" s="5" t="n"/>
-      <c r="F27" s="5" t="n">
+      <c r="E27" s="11" t="n"/>
+      <c r="F27" s="11" t="n">
         <v>75864</v>
       </c>
       <c r="G27" s="2" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="n">
+      <c r="A28" s="9" t="n">
         <v>45994</v>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -5849,17 +5842,17 @@
           <t>100182</t>
         </is>
       </c>
-      <c r="D28" s="5" t="n">
+      <c r="D28" s="11" t="n">
         <v>3857</v>
       </c>
-      <c r="E28" s="5" t="n"/>
-      <c r="F28" s="5" t="n">
+      <c r="E28" s="11" t="n"/>
+      <c r="F28" s="11" t="n">
         <v>72007</v>
       </c>
       <c r="G28" s="2" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="n">
+      <c r="A29" s="9" t="n">
         <v>45999</v>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -5872,17 +5865,17 @@
           <t>100189</t>
         </is>
       </c>
-      <c r="D29" s="5" t="n">
+      <c r="D29" s="11" t="n">
         <v>6524</v>
       </c>
-      <c r="E29" s="5" t="n"/>
-      <c r="F29" s="5" t="n">
+      <c r="E29" s="11" t="n"/>
+      <c r="F29" s="11" t="n">
         <v>65483</v>
       </c>
       <c r="G29" s="2" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="n">
+      <c r="A30" s="9" t="n">
         <v>46001</v>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -5895,19 +5888,19 @@
           <t>100196</t>
         </is>
       </c>
-      <c r="D30" s="5" t="n">
+      <c r="D30" s="11" t="n">
         <v>111</v>
       </c>
-      <c r="E30" s="5" t="n">
+      <c r="E30" s="11" t="n">
         <v>835</v>
       </c>
-      <c r="F30" s="5" t="n">
+      <c r="F30" s="11" t="n">
         <v>66207</v>
       </c>
       <c r="G30" s="2" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="n">
+      <c r="A31" s="9" t="n">
         <v>46004</v>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -5920,17 +5913,17 @@
           <t>100203</t>
         </is>
       </c>
-      <c r="D31" s="5" t="n">
+      <c r="D31" s="11" t="n">
         <v>2448</v>
       </c>
-      <c r="E31" s="5" t="n"/>
-      <c r="F31" s="5" t="n">
+      <c r="E31" s="11" t="n"/>
+      <c r="F31" s="11" t="n">
         <v>63759</v>
       </c>
       <c r="G31" s="2" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="n">
+      <c r="A32" s="9" t="n">
         <v>46008</v>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -5943,17 +5936,17 @@
           <t>100210</t>
         </is>
       </c>
-      <c r="D32" s="5" t="n">
+      <c r="D32" s="11" t="n">
         <v>1240</v>
       </c>
-      <c r="E32" s="5" t="n"/>
-      <c r="F32" s="5" t="n">
+      <c r="E32" s="11" t="n"/>
+      <c r="F32" s="11" t="n">
         <v>62519</v>
       </c>
       <c r="G32" s="2" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="n">
+      <c r="A33" s="9" t="n">
         <v>46013</v>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -5966,17 +5959,17 @@
           <t>100217</t>
         </is>
       </c>
-      <c r="D33" s="5" t="n">
+      <c r="D33" s="11" t="n">
         <v>5037</v>
       </c>
-      <c r="E33" s="5" t="n"/>
-      <c r="F33" s="5" t="n">
+      <c r="E33" s="11" t="n"/>
+      <c r="F33" s="11" t="n">
         <v>57482</v>
       </c>
       <c r="G33" s="2" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="3" t="n">
+      <c r="A34" s="9" t="n">
         <v>46015</v>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -5989,17 +5982,17 @@
           <t>100224</t>
         </is>
       </c>
-      <c r="D34" s="5" t="n">
+      <c r="D34" s="11" t="n">
         <v>714</v>
       </c>
-      <c r="E34" s="5" t="n"/>
-      <c r="F34" s="5" t="n">
+      <c r="E34" s="11" t="n"/>
+      <c r="F34" s="11" t="n">
         <v>56768</v>
       </c>
       <c r="G34" s="2" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="3" t="n">
+      <c r="A35" s="9" t="n">
         <v>46018</v>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -6012,17 +6005,17 @@
           <t>100231</t>
         </is>
       </c>
-      <c r="D35" s="5" t="n">
+      <c r="D35" s="11" t="n">
         <v>2111</v>
       </c>
-      <c r="E35" s="5" t="n"/>
-      <c r="F35" s="5" t="n">
+      <c r="E35" s="11" t="n"/>
+      <c r="F35" s="11" t="n">
         <v>54657</v>
       </c>
       <c r="G35" s="2" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="3" t="n">
+      <c r="A36" s="9" t="n">
         <v>46022</v>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -6035,17 +6028,17 @@
           <t>100238</t>
         </is>
       </c>
-      <c r="D36" s="5" t="n">
+      <c r="D36" s="11" t="n">
         <v>9048</v>
       </c>
-      <c r="E36" s="5" t="n"/>
-      <c r="F36" s="5" t="n">
+      <c r="E36" s="11" t="n"/>
+      <c r="F36" s="11" t="n">
         <v>45609</v>
       </c>
       <c r="G36" s="2" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="3" t="n">
+      <c r="A37" s="9" t="n">
         <v>46027</v>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -6058,17 +6051,17 @@
           <t>100245</t>
         </is>
       </c>
-      <c r="D37" s="5" t="n"/>
-      <c r="E37" s="5" t="n">
+      <c r="D37" s="11" t="n"/>
+      <c r="E37" s="11" t="n">
         <v>122</v>
       </c>
-      <c r="F37" s="5" t="n">
+      <c r="F37" s="11" t="n">
         <v>45731</v>
       </c>
       <c r="G37" s="2" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="3" t="n">
+      <c r="A38" s="9" t="n">
         <v>46029</v>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -6081,19 +6074,19 @@
           <t>100252</t>
         </is>
       </c>
-      <c r="D38" s="5" t="n">
+      <c r="D38" s="11" t="n">
         <v>37</v>
       </c>
-      <c r="E38" s="5" t="n">
+      <c r="E38" s="11" t="n">
         <v>21500</v>
       </c>
-      <c r="F38" s="5" t="n">
+      <c r="F38" s="11" t="n">
         <v>67194</v>
       </c>
       <c r="G38" s="2" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="3" t="n">
+      <c r="A39" s="9" t="n">
         <v>46032</v>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -6106,17 +6099,17 @@
           <t>100259</t>
         </is>
       </c>
-      <c r="D39" s="5" t="n">
+      <c r="D39" s="11" t="n">
         <v>4074</v>
       </c>
-      <c r="E39" s="5" t="n"/>
-      <c r="F39" s="5" t="n">
+      <c r="E39" s="11" t="n"/>
+      <c r="F39" s="11" t="n">
         <v>63120</v>
       </c>
       <c r="G39" s="2" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="3" t="n">
+      <c r="A40" s="9" t="n">
         <v>46036</v>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -6129,17 +6122,17 @@
           <t>100266</t>
         </is>
       </c>
-      <c r="D40" s="5" t="n">
+      <c r="D40" s="11" t="n">
         <v>3931</v>
       </c>
-      <c r="E40" s="5" t="n"/>
-      <c r="F40" s="5" t="n">
+      <c r="E40" s="11" t="n"/>
+      <c r="F40" s="11" t="n">
         <v>59189</v>
       </c>
       <c r="G40" s="2" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="3" t="n">
+      <c r="A41" s="9" t="n">
         <v>46041</v>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -6152,17 +6145,17 @@
           <t>100273</t>
         </is>
       </c>
-      <c r="D41" s="5" t="n">
+      <c r="D41" s="11" t="n">
         <v>6598</v>
       </c>
-      <c r="E41" s="5" t="n"/>
-      <c r="F41" s="5" t="n">
+      <c r="E41" s="11" t="n"/>
+      <c r="F41" s="11" t="n">
         <v>52591</v>
       </c>
       <c r="G41" s="2" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="3" t="n">
+      <c r="A42" s="9" t="n">
         <v>46043</v>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -6175,17 +6168,17 @@
           <t>100280</t>
         </is>
       </c>
-      <c r="D42" s="5" t="n"/>
-      <c r="E42" s="5" t="n">
+      <c r="D42" s="11" t="n"/>
+      <c r="E42" s="11" t="n">
         <v>835</v>
       </c>
-      <c r="F42" s="5" t="n">
+      <c r="F42" s="11" t="n">
         <v>53426</v>
       </c>
       <c r="G42" s="2" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="3" t="n">
+      <c r="A43" s="9" t="n">
         <v>46046</v>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -6198,17 +6191,17 @@
           <t>100287</t>
         </is>
       </c>
-      <c r="D43" s="5" t="n">
+      <c r="D43" s="11" t="n">
         <v>2337</v>
       </c>
-      <c r="E43" s="5" t="n"/>
-      <c r="F43" s="5" t="n">
+      <c r="E43" s="11" t="n"/>
+      <c r="F43" s="11" t="n">
         <v>51089</v>
       </c>
       <c r="G43" s="2" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="3" t="n">
+      <c r="A44" s="9" t="n">
         <v>46050</v>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -6221,17 +6214,17 @@
           <t>100294</t>
         </is>
       </c>
-      <c r="D44" s="5" t="n">
+      <c r="D44" s="11" t="n">
         <v>1314</v>
       </c>
-      <c r="E44" s="5" t="n"/>
-      <c r="F44" s="5" t="n">
+      <c r="E44" s="11" t="n"/>
+      <c r="F44" s="11" t="n">
         <v>49775</v>
       </c>
       <c r="G44" s="2" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="3" t="n">
+      <c r="A45" s="9" t="n">
         <v>46055</v>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -6244,17 +6237,17 @@
           <t>100301</t>
         </is>
       </c>
-      <c r="D45" s="5" t="n">
+      <c r="D45" s="11" t="n">
         <v>5111</v>
       </c>
-      <c r="E45" s="5" t="n"/>
-      <c r="F45" s="5" t="n">
+      <c r="E45" s="11" t="n"/>
+      <c r="F45" s="11" t="n">
         <v>44664</v>
       </c>
       <c r="G45" s="2" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="3" t="n">
+      <c r="A46" s="9" t="n">
         <v>46057</v>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -6267,17 +6260,17 @@
           <t>100308</t>
         </is>
       </c>
-      <c r="D46" s="5" t="n">
+      <c r="D46" s="11" t="n">
         <v>788</v>
       </c>
-      <c r="E46" s="5" t="n"/>
-      <c r="F46" s="5" t="n">
+      <c r="E46" s="11" t="n"/>
+      <c r="F46" s="11" t="n">
         <v>43876</v>
       </c>
       <c r="G46" s="2" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="3" t="n">
+      <c r="A47" s="9" t="n">
         <v>46060</v>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -6290,17 +6283,17 @@
           <t>100315</t>
         </is>
       </c>
-      <c r="D47" s="5" t="n">
+      <c r="D47" s="11" t="n">
         <v>2000</v>
       </c>
-      <c r="E47" s="5" t="n"/>
-      <c r="F47" s="5" t="n">
+      <c r="E47" s="11" t="n"/>
+      <c r="F47" s="11" t="n">
         <v>41876</v>
       </c>
       <c r="G47" s="2" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="3" t="n">
+      <c r="A48" s="9" t="n">
         <v>46064</v>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -6313,17 +6306,17 @@
           <t>100322</t>
         </is>
       </c>
-      <c r="D48" s="5" t="n">
+      <c r="D48" s="11" t="n">
         <v>8937</v>
       </c>
-      <c r="E48" s="5" t="n"/>
-      <c r="F48" s="5" t="n">
+      <c r="E48" s="11" t="n"/>
+      <c r="F48" s="11" t="n">
         <v>32939</v>
       </c>
       <c r="G48" s="2" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="3" t="n">
+      <c r="A49" s="9" t="n">
         <v>46069</v>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -6336,13 +6329,13 @@
           <t>100329</t>
         </is>
       </c>
-      <c r="D49" s="5" t="n">
+      <c r="D49" s="11" t="n">
         <v>74</v>
       </c>
-      <c r="E49" s="5" t="n">
+      <c r="E49" s="11" t="n">
         <v>122</v>
       </c>
-      <c r="F49" s="5" t="n">
+      <c r="F49" s="11" t="n">
         <v>32987</v>
       </c>
       <c r="G49" s="2" t="n"/>
@@ -6422,19 +6415,19 @@
           <t>במעמד חתימת ההסכם</t>
         </is>
       </c>
-      <c r="C2" s="3" t="n">
+      <c r="C2" s="9" t="n">
         <v>45748</v>
       </c>
-      <c r="D2" s="5" t="n">
+      <c r="D2" s="11" t="n">
         <v>250000</v>
       </c>
-      <c r="E2" s="3" t="n">
+      <c r="E2" s="9" t="n">
         <v>45748</v>
       </c>
-      <c r="F2" s="5" t="n">
+      <c r="F2" s="11" t="n">
         <v>250000</v>
       </c>
-      <c r="G2" s="5">
+      <c r="G2" s="11">
         <f>D2-IF(F2="",0,F2)</f>
         <v/>
       </c>
@@ -6449,19 +6442,19 @@
           <t>עם קבלת היתר בנייה</t>
         </is>
       </c>
-      <c r="C3" s="3" t="n">
+      <c r="C3" s="9" t="n">
         <v>45792</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="D3" s="11" t="n">
         <v>400000</v>
       </c>
-      <c r="E3" s="3" t="n">
+      <c r="E3" s="9" t="n">
         <v>45797</v>
       </c>
-      <c r="F3" s="5" t="n">
+      <c r="F3" s="11" t="n">
         <v>400000</v>
       </c>
-      <c r="G3" s="5">
+      <c r="G3" s="11">
         <f>D3-IF(F3="",0,F3)</f>
         <v/>
       </c>
@@ -6476,19 +6469,19 @@
           <t>גמר שלד</t>
         </is>
       </c>
-      <c r="C4" s="3" t="n">
+      <c r="C4" s="9" t="n">
         <v>45870</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="D4" s="11" t="n">
         <v>500000</v>
       </c>
-      <c r="E4" s="3" t="n">
+      <c r="E4" s="9" t="n">
         <v>45872</v>
       </c>
-      <c r="F4" s="5" t="n">
+      <c r="F4" s="11" t="n">
         <v>500000</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="11">
         <f>D4-IF(F4="",0,F4)</f>
         <v/>
       </c>
@@ -6503,19 +6496,19 @@
           <t>גמר טיח וריצוף</t>
         </is>
       </c>
-      <c r="C5" s="3" t="n">
+      <c r="C5" s="9" t="n">
         <v>45962</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="D5" s="11" t="n">
         <v>450000</v>
       </c>
-      <c r="E5" s="3" t="n">
+      <c r="E5" s="9" t="n">
         <v>45989</v>
       </c>
-      <c r="F5" s="5" t="n">
+      <c r="F5" s="11" t="n">
         <v>450000</v>
       </c>
-      <c r="G5" s="5">
+      <c r="G5" s="11">
         <f>D5-IF(F5="",0,F5)</f>
         <v/>
       </c>
@@ -6530,15 +6523,15 @@
           <t>גמר עבודות חשמל ואינסטלציה</t>
         </is>
       </c>
-      <c r="C6" s="3" t="n">
+      <c r="C6" s="9" t="n">
         <v>46037</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="D6" s="11" t="n">
         <v>300000</v>
       </c>
-      <c r="E6" s="3" t="n"/>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5">
+      <c r="E6" s="9" t="n"/>
+      <c r="F6" s="11" t="n"/>
+      <c r="G6" s="11">
         <f>D6-IF(F6="",0,F6)</f>
         <v/>
       </c>
@@ -6553,15 +6546,15 @@
           <t>מסירת החזקה</t>
         </is>
       </c>
-      <c r="C7" s="3" t="n">
+      <c r="C7" s="9" t="n">
         <v>46113</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="D7" s="11" t="n">
         <v>350000</v>
       </c>
-      <c r="E7" s="3" t="n"/>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="5">
+      <c r="E7" s="9" t="n"/>
+      <c r="F7" s="11" t="n"/>
+      <c r="G7" s="11">
         <f>D7-IF(F7="",0,F7)</f>
         <v/>
       </c>
@@ -6576,15 +6569,15 @@
           <t>רישום בטאבו</t>
         </is>
       </c>
-      <c r="C8" s="3" t="n">
+      <c r="C8" s="9" t="n">
         <v>46266</v>
       </c>
-      <c r="D8" s="5" t="n">
+      <c r="D8" s="11" t="n">
         <v>100000</v>
       </c>
-      <c r="E8" s="3" t="n"/>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="5">
+      <c r="E8" s="9" t="n"/>
+      <c r="F8" s="11" t="n"/>
+      <c r="G8" s="11">
         <f>D8-IF(F8="",0,F8)</f>
         <v/>
       </c>

</xml_diff>